<commit_message>
Deploying to gh-pages from  @ 56e8877387266ea804cc7dd83c55667dae371292 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_5-3-1.xlsx
+++ b/assets/excel/2026_5-3-1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69D40CA-97F9-4CEC-B821-A4378F580089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE98992-57ED-4F1A-9FC9-8554ECFE0A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{BEE63AFD-B998-4653-B5B4-F3EC26420D1F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{BEE63AFD-B998-4653-B5B4-F3EC26420D1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -248,10 +248,10 @@
     <t>https://www.integrationsmonitoring.niedersachsen.de</t>
   </si>
   <si>
-    <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2026</t>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                          </t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                          </t>
+    <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2025</t>
   </si>
 </sst>
 </file>
@@ -463,6 +463,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -471,24 +489,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -510,9 +510,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -550,7 +550,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -656,7 +656,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -798,7 +798,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -816,7 +816,7 @@
   <sheetData>
     <row r="1" spans="1:45" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -987,7 +987,7 @@
       <c r="AP5" s="4"/>
     </row>
     <row r="6" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="26" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="17"/>
@@ -997,418 +997,418 @@
       <c r="G6" s="17"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
-      <c r="J6" s="29" t="s">
+      <c r="J6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
-      <c r="O6" s="30"/>
-      <c r="P6" s="30"/>
-      <c r="Q6" s="30"/>
-      <c r="R6" s="30"/>
-      <c r="S6" s="30"/>
-      <c r="T6" s="30"/>
-      <c r="U6" s="30"/>
-      <c r="V6" s="30"/>
-      <c r="W6" s="30"/>
-      <c r="X6" s="30"/>
-      <c r="Y6" s="30"/>
-      <c r="Z6" s="30"/>
-      <c r="AA6" s="30"/>
-      <c r="AB6" s="30"/>
-      <c r="AC6" s="30"/>
-      <c r="AD6" s="30"/>
-      <c r="AE6" s="30"/>
-      <c r="AF6" s="30"/>
-      <c r="AG6" s="30"/>
-      <c r="AH6" s="30"/>
-      <c r="AI6" s="30"/>
-      <c r="AJ6" s="30"/>
-      <c r="AK6" s="30"/>
-      <c r="AL6" s="30"/>
-      <c r="AM6" s="30"/>
-      <c r="AN6" s="30"/>
-      <c r="AO6" s="30"/>
-      <c r="AP6" s="30"/>
-      <c r="AQ6" s="30"/>
-      <c r="AR6" s="30"/>
-      <c r="AS6" s="30"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="28"/>
+      <c r="U6" s="28"/>
+      <c r="V6" s="28"/>
+      <c r="W6" s="28"/>
+      <c r="X6" s="28"/>
+      <c r="Y6" s="28"/>
+      <c r="Z6" s="28"/>
+      <c r="AA6" s="28"/>
+      <c r="AB6" s="28"/>
+      <c r="AC6" s="28"/>
+      <c r="AD6" s="28"/>
+      <c r="AE6" s="28"/>
+      <c r="AF6" s="28"/>
+      <c r="AG6" s="28"/>
+      <c r="AH6" s="28"/>
+      <c r="AI6" s="28"/>
+      <c r="AJ6" s="28"/>
+      <c r="AK6" s="28"/>
+      <c r="AL6" s="28"/>
+      <c r="AM6" s="28"/>
+      <c r="AN6" s="28"/>
+      <c r="AO6" s="28"/>
+      <c r="AP6" s="28"/>
+      <c r="AQ6" s="28"/>
+      <c r="AR6" s="28"/>
+      <c r="AS6" s="28"/>
     </row>
     <row r="7" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="27"/>
-      <c r="C7" s="28" t="s">
+      <c r="B7" s="26"/>
+      <c r="C7" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="24">
         <v>2025</v>
       </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26">
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24">
         <v>2024</v>
       </c>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26">
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24">
         <v>2023</v>
       </c>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26">
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24">
         <v>2022</v>
       </c>
-      <c r="N7" s="26"/>
-      <c r="O7" s="26"/>
-      <c r="P7" s="26">
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24">
         <v>2021</v>
       </c>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="26"/>
-      <c r="S7" s="26" t="s">
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="T7" s="26"/>
-      <c r="U7" s="26"/>
-      <c r="V7" s="26" t="s">
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="W7" s="26"/>
-      <c r="X7" s="26"/>
-      <c r="Y7" s="26" t="s">
+      <c r="W7" s="24"/>
+      <c r="X7" s="24"/>
+      <c r="Y7" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="Z7" s="26"/>
-      <c r="AA7" s="26"/>
-      <c r="AB7" s="26" t="s">
+      <c r="Z7" s="24"/>
+      <c r="AA7" s="24"/>
+      <c r="AB7" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="AC7" s="26"/>
-      <c r="AD7" s="26"/>
-      <c r="AE7" s="26" t="s">
+      <c r="AC7" s="24"/>
+      <c r="AD7" s="24"/>
+      <c r="AE7" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="AF7" s="26"/>
-      <c r="AG7" s="26"/>
-      <c r="AH7" s="26" t="s">
+      <c r="AF7" s="24"/>
+      <c r="AG7" s="24"/>
+      <c r="AH7" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="AI7" s="26"/>
-      <c r="AJ7" s="26"/>
-      <c r="AK7" s="26" t="s">
+      <c r="AI7" s="24"/>
+      <c r="AJ7" s="24"/>
+      <c r="AK7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="AL7" s="26"/>
-      <c r="AM7" s="26"/>
-      <c r="AN7" s="26" t="s">
+      <c r="AL7" s="24"/>
+      <c r="AM7" s="24"/>
+      <c r="AN7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="AO7" s="26"/>
-      <c r="AP7" s="26"/>
-      <c r="AQ7" s="26" t="s">
+      <c r="AO7" s="24"/>
+      <c r="AP7" s="24"/>
+      <c r="AQ7" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="AR7" s="26"/>
-      <c r="AS7" s="29"/>
+      <c r="AR7" s="24"/>
+      <c r="AS7" s="23"/>
     </row>
     <row r="8" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="27"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="26" t="s">
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="H8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="26" t="s">
+      <c r="I8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="26" t="s">
+      <c r="J8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="26" t="s">
+      <c r="K8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="26" t="s">
+      <c r="L8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="26" t="s">
+      <c r="M8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="N8" s="26" t="s">
+      <c r="N8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="O8" s="26" t="s">
+      <c r="O8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="P8" s="26" t="s">
+      <c r="P8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Q8" s="26" t="s">
+      <c r="Q8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="R8" s="26" t="s">
+      <c r="R8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="26" t="s">
+      <c r="S8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="T8" s="26" t="s">
+      <c r="T8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="U8" s="26" t="s">
+      <c r="U8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="26" t="s">
+      <c r="V8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="W8" s="26" t="s">
+      <c r="W8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="X8" s="26" t="s">
+      <c r="X8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="Y8" s="26" t="s">
+      <c r="Y8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Z8" s="26" t="s">
+      <c r="Z8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AA8" s="26" t="s">
+      <c r="AA8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AB8" s="26" t="s">
+      <c r="AB8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AC8" s="26" t="s">
+      <c r="AC8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AD8" s="26" t="s">
+      <c r="AD8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AE8" s="26" t="s">
+      <c r="AE8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AF8" s="26" t="s">
+      <c r="AF8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AG8" s="26" t="s">
+      <c r="AG8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AH8" s="26" t="s">
+      <c r="AH8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AI8" s="26" t="s">
+      <c r="AI8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AJ8" s="26" t="s">
+      <c r="AJ8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AK8" s="26" t="s">
+      <c r="AK8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AL8" s="26" t="s">
+      <c r="AL8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AM8" s="26" t="s">
+      <c r="AM8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AN8" s="26" t="s">
+      <c r="AN8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AO8" s="26" t="s">
+      <c r="AO8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AP8" s="26" t="s">
+      <c r="AP8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="26" t="s">
+      <c r="AQ8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="AR8" s="26" t="s">
+      <c r="AR8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AS8" s="29" t="s">
+      <c r="AS8" s="23" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="27"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="26"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="26"/>
-      <c r="P9" s="26"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="26"/>
-      <c r="T9" s="26"/>
-      <c r="U9" s="26"/>
-      <c r="V9" s="26"/>
-      <c r="W9" s="26"/>
-      <c r="X9" s="26"/>
-      <c r="Y9" s="26"/>
-      <c r="Z9" s="26"/>
-      <c r="AA9" s="26"/>
-      <c r="AB9" s="26"/>
-      <c r="AC9" s="26"/>
-      <c r="AD9" s="26"/>
-      <c r="AE9" s="26"/>
-      <c r="AF9" s="26"/>
-      <c r="AG9" s="26"/>
-      <c r="AH9" s="26"/>
-      <c r="AI9" s="26"/>
-      <c r="AJ9" s="26"/>
-      <c r="AK9" s="26"/>
-      <c r="AL9" s="26"/>
-      <c r="AM9" s="26"/>
-      <c r="AN9" s="26"/>
-      <c r="AO9" s="26"/>
-      <c r="AP9" s="26"/>
-      <c r="AQ9" s="26"/>
-      <c r="AR9" s="26"/>
-      <c r="AS9" s="29"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="24"/>
+      <c r="W9" s="24"/>
+      <c r="X9" s="24"/>
+      <c r="Y9" s="24"/>
+      <c r="Z9" s="24"/>
+      <c r="AA9" s="24"/>
+      <c r="AB9" s="24"/>
+      <c r="AC9" s="24"/>
+      <c r="AD9" s="24"/>
+      <c r="AE9" s="24"/>
+      <c r="AF9" s="24"/>
+      <c r="AG9" s="24"/>
+      <c r="AH9" s="24"/>
+      <c r="AI9" s="24"/>
+      <c r="AJ9" s="24"/>
+      <c r="AK9" s="24"/>
+      <c r="AL9" s="24"/>
+      <c r="AM9" s="24"/>
+      <c r="AN9" s="24"/>
+      <c r="AO9" s="24"/>
+      <c r="AP9" s="24"/>
+      <c r="AQ9" s="24"/>
+      <c r="AR9" s="24"/>
+      <c r="AS9" s="23"/>
     </row>
     <row r="10" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="27"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26" t="s">
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26" t="s">
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26" t="s">
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
-      <c r="N10" s="26" t="s">
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
+      <c r="N10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="O10" s="26"/>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26" t="s">
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="R10" s="26"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="26" t="s">
+      <c r="R10" s="24"/>
+      <c r="S10" s="24"/>
+      <c r="T10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="26"/>
-      <c r="V10" s="26"/>
-      <c r="W10" s="26" t="s">
+      <c r="U10" s="24"/>
+      <c r="V10" s="24"/>
+      <c r="W10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="X10" s="26"/>
-      <c r="Y10" s="26"/>
-      <c r="Z10" s="26" t="s">
+      <c r="X10" s="24"/>
+      <c r="Y10" s="24"/>
+      <c r="Z10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AA10" s="26"/>
-      <c r="AB10" s="26"/>
-      <c r="AC10" s="26" t="s">
+      <c r="AA10" s="24"/>
+      <c r="AB10" s="24"/>
+      <c r="AC10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AD10" s="26"/>
-      <c r="AE10" s="26"/>
-      <c r="AF10" s="26" t="s">
+      <c r="AD10" s="24"/>
+      <c r="AE10" s="24"/>
+      <c r="AF10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AG10" s="26"/>
-      <c r="AH10" s="26"/>
-      <c r="AI10" s="26" t="s">
+      <c r="AG10" s="24"/>
+      <c r="AH10" s="24"/>
+      <c r="AI10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AJ10" s="26"/>
-      <c r="AK10" s="26"/>
-      <c r="AL10" s="26" t="s">
+      <c r="AJ10" s="24"/>
+      <c r="AK10" s="24"/>
+      <c r="AL10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AM10" s="26"/>
-      <c r="AN10" s="26"/>
-      <c r="AO10" s="26" t="s">
+      <c r="AM10" s="24"/>
+      <c r="AN10" s="24"/>
+      <c r="AO10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AP10" s="26"/>
-      <c r="AQ10" s="26"/>
-      <c r="AR10" s="26" t="s">
+      <c r="AP10" s="24"/>
+      <c r="AQ10" s="24"/>
+      <c r="AR10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AS10" s="29"/>
+      <c r="AS10" s="23"/>
     </row>
     <row r="11" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="27"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="31" t="s">
+      <c r="B11" s="26"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="31"/>
-      <c r="M11" s="31"/>
-      <c r="N11" s="31"/>
-      <c r="O11" s="31"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
-      <c r="R11" s="31"/>
-      <c r="S11" s="31"/>
-      <c r="T11" s="31"/>
-      <c r="U11" s="31"/>
-      <c r="V11" s="31"/>
-      <c r="W11" s="31"/>
-      <c r="X11" s="31"/>
-      <c r="Y11" s="31"/>
-      <c r="Z11" s="31"/>
-      <c r="AA11" s="31"/>
-      <c r="AB11" s="31"/>
-      <c r="AC11" s="31"/>
-      <c r="AD11" s="31"/>
-      <c r="AE11" s="31"/>
-      <c r="AF11" s="31"/>
-      <c r="AG11" s="31"/>
-      <c r="AH11" s="31"/>
-      <c r="AI11" s="31"/>
-      <c r="AJ11" s="31"/>
-      <c r="AK11" s="31"/>
-      <c r="AL11" s="31"/>
-      <c r="AM11" s="31"/>
-      <c r="AN11" s="31"/>
-      <c r="AO11" s="31"/>
-      <c r="AP11" s="31"/>
-      <c r="AQ11" s="31"/>
-      <c r="AR11" s="31"/>
-      <c r="AS11" s="31"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="25"/>
+      <c r="R11" s="25"/>
+      <c r="S11" s="25"/>
+      <c r="T11" s="25"/>
+      <c r="U11" s="25"/>
+      <c r="V11" s="25"/>
+      <c r="W11" s="25"/>
+      <c r="X11" s="25"/>
+      <c r="Y11" s="25"/>
+      <c r="Z11" s="25"/>
+      <c r="AA11" s="25"/>
+      <c r="AB11" s="25"/>
+      <c r="AC11" s="25"/>
+      <c r="AD11" s="25"/>
+      <c r="AE11" s="25"/>
+      <c r="AF11" s="25"/>
+      <c r="AG11" s="25"/>
+      <c r="AH11" s="25"/>
+      <c r="AI11" s="25"/>
+      <c r="AJ11" s="25"/>
+      <c r="AK11" s="25"/>
+      <c r="AL11" s="25"/>
+      <c r="AM11" s="25"/>
+      <c r="AN11" s="25"/>
+      <c r="AO11" s="25"/>
+      <c r="AP11" s="25"/>
+      <c r="AQ11" s="25"/>
+      <c r="AR11" s="25"/>
+      <c r="AS11" s="25"/>
     </row>
     <row r="12" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="18">
@@ -1556,10 +1556,10 @@
         <v>3.9</v>
       </c>
       <c r="E13" s="15">
+        <v>3.26</v>
+      </c>
+      <c r="F13" s="15">
         <v>5.01</v>
-      </c>
-      <c r="F13" s="15">
-        <v>3.26</v>
       </c>
       <c r="G13" s="15">
         <v>3.77</v>
@@ -1691,10 +1691,10 @@
         <v>4.08</v>
       </c>
       <c r="E14" s="15">
+        <v>2.81</v>
+      </c>
+      <c r="F14" s="15">
         <v>6.73</v>
-      </c>
-      <c r="F14" s="15">
-        <v>2.81</v>
       </c>
       <c r="G14" s="15">
         <v>3.32</v>
@@ -1826,10 +1826,10 @@
         <v>2.92</v>
       </c>
       <c r="E15" s="15">
+        <v>1.84</v>
+      </c>
+      <c r="F15" s="15">
         <v>4.96</v>
-      </c>
-      <c r="F15" s="15">
-        <v>1.84</v>
       </c>
       <c r="G15" s="15">
         <v>2.6</v>
@@ -1961,10 +1961,10 @@
         <v>2.1</v>
       </c>
       <c r="E16" s="15">
+        <v>1.28</v>
+      </c>
+      <c r="F16" s="15">
         <v>4.0599999999999996</v>
-      </c>
-      <c r="F16" s="15">
-        <v>1.28</v>
       </c>
       <c r="G16" s="15">
         <v>1.89</v>
@@ -2096,10 +2096,10 @@
         <v>1.68</v>
       </c>
       <c r="E17" s="15">
+        <v>1.49</v>
+      </c>
+      <c r="F17" s="15">
         <v>2.64</v>
-      </c>
-      <c r="F17" s="15">
-        <v>1.49</v>
       </c>
       <c r="G17" s="15">
         <v>1.57</v>
@@ -2231,10 +2231,10 @@
         <v>2.84</v>
       </c>
       <c r="E18" s="15">
+        <v>2.02</v>
+      </c>
+      <c r="F18" s="15">
         <v>4.8499999999999996</v>
-      </c>
-      <c r="F18" s="15">
-        <v>2.02</v>
       </c>
       <c r="G18" s="15">
         <v>2.54</v>
@@ -2366,10 +2366,10 @@
         <v>4.21</v>
       </c>
       <c r="E19" s="15">
+        <v>3.52</v>
+      </c>
+      <c r="F19" s="15">
         <v>5.35</v>
-      </c>
-      <c r="F19" s="15">
-        <v>3.52</v>
       </c>
       <c r="G19" s="15">
         <v>3.85</v>
@@ -2501,10 +2501,10 @@
         <v>4.75</v>
       </c>
       <c r="E20" s="15">
+        <v>3.34</v>
+      </c>
+      <c r="F20" s="15">
         <v>7.56</v>
-      </c>
-      <c r="F20" s="15">
-        <v>3.34</v>
       </c>
       <c r="G20" s="15">
         <v>3.71</v>
@@ -2636,10 +2636,10 @@
         <v>3.34</v>
       </c>
       <c r="E21" s="15">
+        <v>1.85</v>
+      </c>
+      <c r="F21" s="15">
         <v>6.08</v>
-      </c>
-      <c r="F21" s="15">
-        <v>1.85</v>
       </c>
       <c r="G21" s="15">
         <v>2.69</v>
@@ -2771,10 +2771,10 @@
         <v>2.4300000000000002</v>
       </c>
       <c r="E22" s="15">
+        <v>1.62</v>
+      </c>
+      <c r="F22" s="15">
         <v>4.4000000000000004</v>
-      </c>
-      <c r="F22" s="15">
-        <v>1.62</v>
       </c>
       <c r="G22" s="15">
         <v>2</v>
@@ -2906,10 +2906,10 @@
         <v>2.04</v>
       </c>
       <c r="E23" s="15">
+        <v>1.73</v>
+      </c>
+      <c r="F23" s="15">
         <v>3.6</v>
-      </c>
-      <c r="F23" s="15">
-        <v>1.73</v>
       </c>
       <c r="G23" s="15">
         <v>1.76</v>
@@ -3041,10 +3041,10 @@
         <v>3.29</v>
       </c>
       <c r="E24" s="15">
+        <v>2.31</v>
+      </c>
+      <c r="F24" s="15">
         <v>5.63</v>
-      </c>
-      <c r="F24" s="15">
-        <v>2.31</v>
       </c>
       <c r="G24" s="15">
         <v>2.74</v>
@@ -3176,10 +3176,10 @@
         <v>3.57</v>
       </c>
       <c r="E25" s="15">
+        <v>2.98</v>
+      </c>
+      <c r="F25" s="15">
         <v>4.62</v>
-      </c>
-      <c r="F25" s="15">
-        <v>2.98</v>
       </c>
       <c r="G25" s="15">
         <v>3.68</v>
@@ -3311,10 +3311,10 @@
         <v>3.36</v>
       </c>
       <c r="E26" s="15">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="F26" s="15">
         <v>5.78</v>
-      </c>
-      <c r="F26" s="15">
-        <v>2.2400000000000002</v>
       </c>
       <c r="G26" s="15">
         <v>2.91</v>
@@ -3446,10 +3446,10 @@
         <v>2.5</v>
       </c>
       <c r="E27" s="15">
+        <v>1.83</v>
+      </c>
+      <c r="F27" s="15">
         <v>3.79</v>
-      </c>
-      <c r="F27" s="15">
-        <v>1.83</v>
       </c>
       <c r="G27" s="15">
         <v>2.5</v>
@@ -3581,10 +3581,10 @@
         <v>1.78</v>
       </c>
       <c r="E28" s="15">
+        <v>0.95</v>
+      </c>
+      <c r="F28" s="15">
         <v>3.73</v>
-      </c>
-      <c r="F28" s="15">
-        <v>0.95</v>
       </c>
       <c r="G28" s="15">
         <v>1.78</v>
@@ -3716,10 +3716,10 @@
         <v>1.34</v>
       </c>
       <c r="E29" s="15">
+        <v>1.26</v>
+      </c>
+      <c r="F29" s="15">
         <v>1.73</v>
-      </c>
-      <c r="F29" s="15">
-        <v>1.26</v>
       </c>
       <c r="G29" s="15">
         <v>1.38</v>
@@ -3851,10 +3851,10 @@
         <v>2.39</v>
       </c>
       <c r="E30" s="15">
+        <v>1.73</v>
+      </c>
+      <c r="F30" s="15">
         <v>4.03</v>
-      </c>
-      <c r="F30" s="15">
-        <v>1.73</v>
       </c>
       <c r="G30" s="15">
         <v>2.35</v>
@@ -3978,91 +3978,91 @@
       <c r="B31" s="7"/>
     </row>
     <row r="32" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="23"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="23"/>
-      <c r="T32" s="23"/>
-      <c r="U32" s="23"/>
-      <c r="V32" s="23"/>
-      <c r="W32" s="23"/>
-      <c r="X32" s="23"/>
-      <c r="Y32" s="23"/>
-      <c r="Z32" s="23"/>
-      <c r="AA32" s="23"/>
-      <c r="AB32" s="23"/>
-      <c r="AC32" s="23"/>
-      <c r="AD32" s="23"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="29"/>
+      <c r="P32" s="29"/>
+      <c r="Q32" s="29"/>
+      <c r="R32" s="29"/>
+      <c r="S32" s="29"/>
+      <c r="T32" s="29"/>
+      <c r="U32" s="29"/>
+      <c r="V32" s="29"/>
+      <c r="W32" s="29"/>
+      <c r="X32" s="29"/>
+      <c r="Y32" s="29"/>
+      <c r="Z32" s="29"/>
+      <c r="AA32" s="29"/>
+      <c r="AB32" s="29"/>
+      <c r="AC32" s="29"/>
+      <c r="AD32" s="29"/>
     </row>
     <row r="33" spans="2:30" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
-      <c r="K33" s="24"/>
-      <c r="L33" s="24"/>
-      <c r="M33" s="24"/>
-      <c r="N33" s="24"/>
-      <c r="O33" s="24"/>
-      <c r="P33" s="24"/>
-      <c r="Q33" s="24"/>
-      <c r="R33" s="24"/>
-      <c r="S33" s="24"/>
-      <c r="T33" s="24"/>
-      <c r="U33" s="24"/>
-      <c r="V33" s="24"/>
-      <c r="W33" s="24"/>
-      <c r="X33" s="24"/>
-      <c r="Y33" s="24"/>
-      <c r="Z33" s="24"/>
-      <c r="AA33" s="24"/>
-      <c r="AB33" s="24"/>
-      <c r="AC33" s="24"/>
-      <c r="AD33" s="24"/>
+      <c r="C33" s="30"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="30"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="30"/>
+      <c r="O33" s="30"/>
+      <c r="P33" s="30"/>
+      <c r="Q33" s="30"/>
+      <c r="R33" s="30"/>
+      <c r="S33" s="30"/>
+      <c r="T33" s="30"/>
+      <c r="U33" s="30"/>
+      <c r="V33" s="30"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="30"/>
+      <c r="Y33" s="30"/>
+      <c r="Z33" s="30"/>
+      <c r="AA33" s="30"/>
+      <c r="AB33" s="30"/>
+      <c r="AC33" s="30"/>
+      <c r="AD33" s="30"/>
     </row>
     <row r="34" spans="2:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="25"/>
-      <c r="J34" s="25"/>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
-      <c r="O34" s="25"/>
-      <c r="P34" s="25"/>
-      <c r="Q34" s="25"/>
-      <c r="R34" s="25"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="31"/>
+      <c r="O34" s="31"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="31"/>
     </row>
     <row r="35" spans="2:30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="10" t="s">
@@ -4156,7 +4156,7 @@
     </row>
     <row r="40" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B40" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="2:30" x14ac:dyDescent="0.25">
@@ -4171,6 +4171,67 @@
     </row>
   </sheetData>
   <mergeCells count="77">
+    <mergeCell ref="B32:AD32"/>
+    <mergeCell ref="B33:AD33"/>
+    <mergeCell ref="B34:R34"/>
+    <mergeCell ref="AN8:AN10"/>
+    <mergeCell ref="AO8:AO9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="W10:X10"/>
+    <mergeCell ref="AH8:AH10"/>
+    <mergeCell ref="AL8:AL9"/>
+    <mergeCell ref="AM8:AM9"/>
+    <mergeCell ref="AI10:AJ10"/>
+    <mergeCell ref="AL10:AM10"/>
+    <mergeCell ref="AO10:AP10"/>
+    <mergeCell ref="AP8:AP9"/>
+    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="AF8:AF9"/>
+    <mergeCell ref="AI8:AI9"/>
+    <mergeCell ref="AJ8:AJ9"/>
+    <mergeCell ref="AK8:AK10"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S10"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="AG8:AG9"/>
+    <mergeCell ref="AC10:AD10"/>
+    <mergeCell ref="AF10:AG10"/>
+    <mergeCell ref="V8:V10"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y10"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="AB8:AB10"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="B6:B11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J6:AS6"/>
+    <mergeCell ref="AQ7:AS7"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AR8:AR9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="Y7:AA7"/>
+    <mergeCell ref="AB7:AD7"/>
+    <mergeCell ref="AE7:AG7"/>
+    <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E9"/>
     <mergeCell ref="AS8:AS9"/>
     <mergeCell ref="AR10:AS10"/>
     <mergeCell ref="D11:AS11"/>
@@ -4187,67 +4248,6 @@
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="B6:B11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J6:AS6"/>
-    <mergeCell ref="AQ7:AS7"/>
-    <mergeCell ref="AQ8:AQ10"/>
-    <mergeCell ref="AR8:AR9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="Y7:AA7"/>
-    <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="AE7:AG7"/>
-    <mergeCell ref="AH7:AJ7"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S10"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="AG8:AG9"/>
-    <mergeCell ref="AC10:AD10"/>
-    <mergeCell ref="AF10:AG10"/>
-    <mergeCell ref="V8:V10"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y10"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="AB8:AB10"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="AL10:AM10"/>
-    <mergeCell ref="AO10:AP10"/>
-    <mergeCell ref="AP8:AP9"/>
-    <mergeCell ref="AE8:AE10"/>
-    <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="AI8:AI9"/>
-    <mergeCell ref="AJ8:AJ9"/>
-    <mergeCell ref="AK8:AK10"/>
-    <mergeCell ref="B32:AD32"/>
-    <mergeCell ref="B33:AD33"/>
-    <mergeCell ref="B34:R34"/>
-    <mergeCell ref="AN8:AN10"/>
-    <mergeCell ref="AO8:AO9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="W10:X10"/>
-    <mergeCell ref="AH8:AH10"/>
-    <mergeCell ref="AL8:AL9"/>
-    <mergeCell ref="AM8:AM9"/>
-    <mergeCell ref="AI10:AJ10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B42" r:id="rId1" xr:uid="{F94324D3-9937-4F3E-A4F8-7AD7EC469BFB}"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 7ca7789cd0edf32eab25d1ff5d7f0c46abd765fb 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_5-3-1.xlsx
+++ b/assets/excel/2026_5-3-1.xlsx
@@ -5,17 +5,17 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE98992-57ED-4F1A-9FC9-8554ECFE0A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63F7078-BF64-4BAE-8AA2-32C521B7C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{BEE63AFD-B998-4653-B5B4-F3EC26420D1F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{BEE63AFD-B998-4653-B5B4-F3EC26420D1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -223,16 +223,6 @@
     <t>Frauen</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Hochrechnung anhand der Bevölkerungsfortschreibung auf Basis des Zensus 2011. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 Umstellung erfolgte die auf eine neue Mikrozensus-Stichprobe. Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Durch eine rückwirkende Revision der Mikrozensusdaten wird auch für das Jahr 2017 der Migrationshintergrund im weiteren Sinne dargestellt. Die in den Tabellen ab dem Jahr 2017 berichteten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2016 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit zwischen den Jahren ist dadurch eingeschränkt.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes: </t>
-  </si>
-  <si>
     <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
   </si>
   <si>
@@ -248,10 +238,19 @@
     <t>https://www.integrationsmonitoring.niedersachsen.de</t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                          </t>
+    <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2025</t>
   </si>
   <si>
-    <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2025</t>
+    <t>1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
@@ -261,7 +260,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +312,11 @@
       <u/>
       <sz val="6"/>
       <color theme="10"/>
+      <name val="NDSFrutiger 45 Light"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color theme="1"/>
       <name val="NDSFrutiger 45 Light"/>
     </font>
   </fonts>
@@ -399,7 +403,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -423,23 +427,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -463,13 +452,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -478,18 +464,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -816,7 +804,7 @@
   <sheetData>
     <row r="1" spans="1:45" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -986,3215 +974,3211 @@
       <c r="AM5" s="5"/>
       <c r="AP5" s="4"/>
     </row>
-    <row r="6" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="26" t="s">
+    <row r="6" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="23" t="s">
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28"/>
-      <c r="T6" s="28"/>
-      <c r="U6" s="28"/>
-      <c r="V6" s="28"/>
-      <c r="W6" s="28"/>
-      <c r="X6" s="28"/>
-      <c r="Y6" s="28"/>
-      <c r="Z6" s="28"/>
-      <c r="AA6" s="28"/>
-      <c r="AB6" s="28"/>
-      <c r="AC6" s="28"/>
-      <c r="AD6" s="28"/>
-      <c r="AE6" s="28"/>
-      <c r="AF6" s="28"/>
-      <c r="AG6" s="28"/>
-      <c r="AH6" s="28"/>
-      <c r="AI6" s="28"/>
-      <c r="AJ6" s="28"/>
-      <c r="AK6" s="28"/>
-      <c r="AL6" s="28"/>
-      <c r="AM6" s="28"/>
-      <c r="AN6" s="28"/>
-      <c r="AO6" s="28"/>
-      <c r="AP6" s="28"/>
-      <c r="AQ6" s="28"/>
-      <c r="AR6" s="28"/>
-      <c r="AS6" s="28"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="23"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="23"/>
+      <c r="X6" s="23"/>
+      <c r="Y6" s="23"/>
+      <c r="Z6" s="23"/>
+      <c r="AA6" s="23"/>
+      <c r="AB6" s="23"/>
+      <c r="AC6" s="23"/>
+      <c r="AD6" s="23"/>
+      <c r="AE6" s="23"/>
+      <c r="AF6" s="23"/>
+      <c r="AG6" s="23"/>
+      <c r="AH6" s="23"/>
+      <c r="AI6" s="23"/>
+      <c r="AJ6" s="23"/>
+      <c r="AK6" s="23"/>
+      <c r="AL6" s="23"/>
+      <c r="AM6" s="23"/>
+      <c r="AN6" s="23"/>
+      <c r="AO6" s="23"/>
+      <c r="AP6" s="23"/>
+      <c r="AQ6" s="23"/>
+      <c r="AR6" s="23"/>
+      <c r="AS6" s="23"/>
     </row>
-    <row r="7" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="26"/>
-      <c r="C7" s="27" t="s">
+    <row r="7" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="20"/>
+      <c r="C7" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="19">
         <v>2025</v>
       </c>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24">
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19">
         <v>2024</v>
       </c>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24">
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19">
         <v>2023</v>
       </c>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24">
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19">
         <v>2022</v>
       </c>
-      <c r="N7" s="24"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24">
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19">
         <v>2021</v>
       </c>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="24"/>
-      <c r="S7" s="24" t="s">
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="T7" s="24"/>
-      <c r="U7" s="24"/>
-      <c r="V7" s="24" t="s">
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="W7" s="24"/>
-      <c r="X7" s="24"/>
-      <c r="Y7" s="24" t="s">
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
+      <c r="Y7" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="Z7" s="24"/>
-      <c r="AA7" s="24"/>
-      <c r="AB7" s="24" t="s">
+      <c r="Z7" s="19"/>
+      <c r="AA7" s="19"/>
+      <c r="AB7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="AC7" s="24"/>
-      <c r="AD7" s="24"/>
-      <c r="AE7" s="24" t="s">
+      <c r="AC7" s="19"/>
+      <c r="AD7" s="19"/>
+      <c r="AE7" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="AF7" s="24"/>
-      <c r="AG7" s="24"/>
-      <c r="AH7" s="24" t="s">
+      <c r="AF7" s="19"/>
+      <c r="AG7" s="19"/>
+      <c r="AH7" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="AI7" s="24"/>
-      <c r="AJ7" s="24"/>
-      <c r="AK7" s="24" t="s">
+      <c r="AI7" s="19"/>
+      <c r="AJ7" s="19"/>
+      <c r="AK7" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="AL7" s="24"/>
-      <c r="AM7" s="24"/>
-      <c r="AN7" s="24" t="s">
+      <c r="AL7" s="19"/>
+      <c r="AM7" s="19"/>
+      <c r="AN7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="AO7" s="24"/>
-      <c r="AP7" s="24"/>
-      <c r="AQ7" s="24" t="s">
+      <c r="AO7" s="19"/>
+      <c r="AP7" s="19"/>
+      <c r="AQ7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="AR7" s="24"/>
-      <c r="AS7" s="23"/>
+      <c r="AR7" s="19"/>
+      <c r="AS7" s="22"/>
     </row>
-    <row r="8" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="26"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="24" t="s">
+    <row r="8" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="20"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="I8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="24" t="s">
+      <c r="J8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="24" t="s">
+      <c r="K8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="24" t="s">
+      <c r="L8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="24" t="s">
+      <c r="M8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="N8" s="24" t="s">
+      <c r="N8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O8" s="24" t="s">
+      <c r="O8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="P8" s="24" t="s">
+      <c r="P8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="Q8" s="24" t="s">
+      <c r="Q8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="R8" s="24" t="s">
+      <c r="R8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="24" t="s">
+      <c r="S8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="T8" s="24" t="s">
+      <c r="T8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="U8" s="24" t="s">
+      <c r="U8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="24" t="s">
+      <c r="V8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="W8" s="24" t="s">
+      <c r="W8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="X8" s="24" t="s">
+      <c r="X8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="Y8" s="24" t="s">
+      <c r="Y8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="Z8" s="24" t="s">
+      <c r="Z8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AA8" s="24" t="s">
+      <c r="AA8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AB8" s="24" t="s">
+      <c r="AB8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AC8" s="24" t="s">
+      <c r="AC8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AD8" s="24" t="s">
+      <c r="AD8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AE8" s="24" t="s">
+      <c r="AE8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AF8" s="24" t="s">
+      <c r="AF8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AG8" s="24" t="s">
+      <c r="AG8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AH8" s="24" t="s">
+      <c r="AH8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AI8" s="24" t="s">
+      <c r="AI8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AJ8" s="24" t="s">
+      <c r="AJ8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AK8" s="24" t="s">
+      <c r="AK8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AL8" s="24" t="s">
+      <c r="AL8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AM8" s="24" t="s">
+      <c r="AM8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AN8" s="24" t="s">
+      <c r="AN8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AO8" s="24" t="s">
+      <c r="AO8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AP8" s="24" t="s">
+      <c r="AP8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="24" t="s">
+      <c r="AQ8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="AR8" s="24" t="s">
+      <c r="AR8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AS8" s="23" t="s">
+      <c r="AS8" s="22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="26"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
-      <c r="L9" s="24"/>
-      <c r="M9" s="24"/>
-      <c r="N9" s="24"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="24"/>
-      <c r="S9" s="24"/>
-      <c r="T9" s="24"/>
-      <c r="U9" s="24"/>
-      <c r="V9" s="24"/>
-      <c r="W9" s="24"/>
-      <c r="X9" s="24"/>
-      <c r="Y9" s="24"/>
-      <c r="Z9" s="24"/>
-      <c r="AA9" s="24"/>
-      <c r="AB9" s="24"/>
-      <c r="AC9" s="24"/>
-      <c r="AD9" s="24"/>
-      <c r="AE9" s="24"/>
-      <c r="AF9" s="24"/>
-      <c r="AG9" s="24"/>
-      <c r="AH9" s="24"/>
-      <c r="AI9" s="24"/>
-      <c r="AJ9" s="24"/>
-      <c r="AK9" s="24"/>
-      <c r="AL9" s="24"/>
-      <c r="AM9" s="24"/>
-      <c r="AN9" s="24"/>
-      <c r="AO9" s="24"/>
-      <c r="AP9" s="24"/>
-      <c r="AQ9" s="24"/>
-      <c r="AR9" s="24"/>
-      <c r="AS9" s="23"/>
+    <row r="9" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="19"/>
+      <c r="AA9" s="19"/>
+      <c r="AB9" s="19"/>
+      <c r="AC9" s="19"/>
+      <c r="AD9" s="19"/>
+      <c r="AE9" s="19"/>
+      <c r="AF9" s="19"/>
+      <c r="AG9" s="19"/>
+      <c r="AH9" s="19"/>
+      <c r="AI9" s="19"/>
+      <c r="AJ9" s="19"/>
+      <c r="AK9" s="19"/>
+      <c r="AL9" s="19"/>
+      <c r="AM9" s="19"/>
+      <c r="AN9" s="19"/>
+      <c r="AO9" s="19"/>
+      <c r="AP9" s="19"/>
+      <c r="AQ9" s="19"/>
+      <c r="AR9" s="19"/>
+      <c r="AS9" s="22"/>
     </row>
-    <row r="10" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="26"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24" t="s">
+    <row r="10" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="20"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24" t="s">
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24" t="s">
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24" t="s">
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24" t="s">
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="R10" s="24"/>
-      <c r="S10" s="24"/>
-      <c r="T10" s="24" t="s">
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="24"/>
-      <c r="V10" s="24"/>
-      <c r="W10" s="24" t="s">
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="X10" s="24"/>
-      <c r="Y10" s="24"/>
-      <c r="Z10" s="24" t="s">
+      <c r="X10" s="19"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AA10" s="24"/>
-      <c r="AB10" s="24"/>
-      <c r="AC10" s="24" t="s">
+      <c r="AA10" s="19"/>
+      <c r="AB10" s="19"/>
+      <c r="AC10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AD10" s="24"/>
-      <c r="AE10" s="24"/>
-      <c r="AF10" s="24" t="s">
+      <c r="AD10" s="19"/>
+      <c r="AE10" s="19"/>
+      <c r="AF10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AG10" s="24"/>
-      <c r="AH10" s="24"/>
-      <c r="AI10" s="24" t="s">
+      <c r="AG10" s="19"/>
+      <c r="AH10" s="19"/>
+      <c r="AI10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AJ10" s="24"/>
-      <c r="AK10" s="24"/>
-      <c r="AL10" s="24" t="s">
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="19"/>
+      <c r="AL10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AM10" s="24"/>
-      <c r="AN10" s="24"/>
-      <c r="AO10" s="24" t="s">
+      <c r="AM10" s="19"/>
+      <c r="AN10" s="19"/>
+      <c r="AO10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AP10" s="24"/>
-      <c r="AQ10" s="24"/>
-      <c r="AR10" s="24" t="s">
+      <c r="AP10" s="19"/>
+      <c r="AQ10" s="19"/>
+      <c r="AR10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="AS10" s="23"/>
+      <c r="AS10" s="22"/>
     </row>
-    <row r="11" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="26"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="25" t="s">
+    <row r="11" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="20"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="25"/>
-      <c r="U11" s="25"/>
-      <c r="V11" s="25"/>
-      <c r="W11" s="25"/>
-      <c r="X11" s="25"/>
-      <c r="Y11" s="25"/>
-      <c r="Z11" s="25"/>
-      <c r="AA11" s="25"/>
-      <c r="AB11" s="25"/>
-      <c r="AC11" s="25"/>
-      <c r="AD11" s="25"/>
-      <c r="AE11" s="25"/>
-      <c r="AF11" s="25"/>
-      <c r="AG11" s="25"/>
-      <c r="AH11" s="25"/>
-      <c r="AI11" s="25"/>
-      <c r="AJ11" s="25"/>
-      <c r="AK11" s="25"/>
-      <c r="AL11" s="25"/>
-      <c r="AM11" s="25"/>
-      <c r="AN11" s="25"/>
-      <c r="AO11" s="25"/>
-      <c r="AP11" s="25"/>
-      <c r="AQ11" s="25"/>
-      <c r="AR11" s="25"/>
-      <c r="AS11" s="25"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24"/>
+      <c r="T11" s="24"/>
+      <c r="U11" s="24"/>
+      <c r="V11" s="24"/>
+      <c r="W11" s="24"/>
+      <c r="X11" s="24"/>
+      <c r="Y11" s="24"/>
+      <c r="Z11" s="24"/>
+      <c r="AA11" s="24"/>
+      <c r="AB11" s="24"/>
+      <c r="AC11" s="24"/>
+      <c r="AD11" s="24"/>
+      <c r="AE11" s="24"/>
+      <c r="AF11" s="24"/>
+      <c r="AG11" s="24"/>
+      <c r="AH11" s="24"/>
+      <c r="AI11" s="24"/>
+      <c r="AJ11" s="24"/>
+      <c r="AK11" s="24"/>
+      <c r="AL11" s="24"/>
+      <c r="AM11" s="24"/>
+      <c r="AN11" s="24"/>
+      <c r="AO11" s="24"/>
+      <c r="AP11" s="24"/>
+      <c r="AQ11" s="24"/>
+      <c r="AR11" s="24"/>
+      <c r="AS11" s="24"/>
     </row>
-    <row r="12" spans="1:45" s="16" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="18">
+    <row r="12" spans="1:45" s="11" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="13">
         <v>1</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="13">
         <v>2</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="13">
         <v>3</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="13">
         <v>4</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="13">
         <v>5</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="13">
         <v>6</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="13">
         <v>7</v>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="13">
         <v>8</v>
       </c>
-      <c r="J12" s="18">
+      <c r="J12" s="13">
         <v>9</v>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="13">
         <v>10</v>
       </c>
-      <c r="L12" s="18">
+      <c r="L12" s="13">
         <v>11</v>
       </c>
-      <c r="M12" s="18">
+      <c r="M12" s="13">
         <v>12</v>
       </c>
-      <c r="N12" s="18">
+      <c r="N12" s="13">
         <v>13</v>
       </c>
-      <c r="O12" s="18">
+      <c r="O12" s="13">
         <v>14</v>
       </c>
-      <c r="P12" s="18">
+      <c r="P12" s="13">
         <v>15</v>
       </c>
-      <c r="Q12" s="18">
+      <c r="Q12" s="13">
         <v>16</v>
       </c>
-      <c r="R12" s="18">
+      <c r="R12" s="13">
         <v>17</v>
       </c>
-      <c r="S12" s="18">
+      <c r="S12" s="13">
         <v>18</v>
       </c>
-      <c r="T12" s="18">
+      <c r="T12" s="13">
         <v>19</v>
       </c>
-      <c r="U12" s="18">
+      <c r="U12" s="13">
         <v>20</v>
       </c>
-      <c r="V12" s="18">
+      <c r="V12" s="13">
         <v>21</v>
       </c>
-      <c r="W12" s="18">
+      <c r="W12" s="13">
         <v>22</v>
       </c>
-      <c r="X12" s="18">
+      <c r="X12" s="13">
         <v>23</v>
       </c>
-      <c r="Y12" s="18">
+      <c r="Y12" s="13">
         <v>24</v>
       </c>
-      <c r="Z12" s="18">
+      <c r="Z12" s="13">
         <v>25</v>
       </c>
-      <c r="AA12" s="18">
+      <c r="AA12" s="13">
         <v>26</v>
       </c>
-      <c r="AB12" s="18">
+      <c r="AB12" s="13">
         <v>27</v>
       </c>
-      <c r="AC12" s="18">
+      <c r="AC12" s="13">
         <v>28</v>
       </c>
-      <c r="AD12" s="18">
+      <c r="AD12" s="13">
         <v>29</v>
       </c>
-      <c r="AE12" s="18">
+      <c r="AE12" s="13">
         <v>30</v>
       </c>
-      <c r="AF12" s="18">
+      <c r="AF12" s="13">
         <v>31</v>
       </c>
-      <c r="AG12" s="18">
+      <c r="AG12" s="13">
         <v>32</v>
       </c>
-      <c r="AH12" s="18">
+      <c r="AH12" s="13">
         <v>33</v>
       </c>
-      <c r="AI12" s="18">
+      <c r="AI12" s="13">
         <v>34</v>
       </c>
-      <c r="AJ12" s="18">
+      <c r="AJ12" s="13">
         <v>35</v>
       </c>
-      <c r="AK12" s="18">
+      <c r="AK12" s="13">
         <v>36</v>
       </c>
-      <c r="AL12" s="18">
+      <c r="AL12" s="13">
         <v>37</v>
       </c>
-      <c r="AM12" s="18">
+      <c r="AM12" s="13">
         <v>38</v>
       </c>
-      <c r="AN12" s="18">
+      <c r="AN12" s="13">
         <v>39</v>
       </c>
-      <c r="AO12" s="18">
+      <c r="AO12" s="13">
         <v>40</v>
       </c>
-      <c r="AP12" s="18">
+      <c r="AP12" s="13">
         <v>41</v>
       </c>
-      <c r="AQ12" s="18">
+      <c r="AQ12" s="13">
         <v>42</v>
       </c>
-      <c r="AR12" s="18">
+      <c r="AR12" s="13">
         <v>43</v>
       </c>
-      <c r="AS12" s="18">
+      <c r="AS12" s="13">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="20" t="s">
+    <row r="13" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="10">
         <v>3.9</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="10">
         <v>3.26</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="10">
         <v>5.01</v>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="10">
         <v>3.77</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="10">
         <v>3.33</v>
       </c>
-      <c r="I13" s="15">
+      <c r="I13" s="10">
         <v>4.58</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="10">
         <v>3.33</v>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="10">
         <v>2.83</v>
       </c>
-      <c r="L13" s="15">
+      <c r="L13" s="10">
         <v>4.34</v>
       </c>
-      <c r="M13" s="15">
+      <c r="M13" s="10">
         <v>2.94</v>
       </c>
-      <c r="N13" s="15">
+      <c r="N13" s="10">
         <v>2.68</v>
       </c>
-      <c r="O13" s="15">
+      <c r="O13" s="10">
         <v>3.51</v>
       </c>
-      <c r="P13" s="15">
+      <c r="P13" s="10">
         <v>3.42</v>
       </c>
-      <c r="Q13" s="15">
+      <c r="Q13" s="10">
         <v>3.07</v>
       </c>
-      <c r="R13" s="15">
+      <c r="R13" s="10">
         <v>4.2699999999999996</v>
       </c>
-      <c r="S13" s="15">
+      <c r="S13" s="10">
         <v>3.21</v>
       </c>
-      <c r="T13" s="15">
+      <c r="T13" s="10">
         <v>2.6</v>
       </c>
-      <c r="U13" s="15">
+      <c r="U13" s="10">
         <v>4.78</v>
       </c>
-      <c r="V13" s="15">
+      <c r="V13" s="10">
         <v>3.15</v>
       </c>
-      <c r="W13" s="15">
+      <c r="W13" s="10">
         <v>2.82</v>
       </c>
-      <c r="X13" s="15">
+      <c r="X13" s="10">
         <v>4.03</v>
       </c>
-      <c r="Y13" s="15">
+      <c r="Y13" s="10">
         <v>3.15</v>
       </c>
-      <c r="Z13" s="15">
+      <c r="Z13" s="10">
         <v>2.4900000000000002</v>
       </c>
-      <c r="AA13" s="15">
+      <c r="AA13" s="10">
         <v>4.84</v>
       </c>
-      <c r="AB13" s="15">
+      <c r="AB13" s="10">
         <v>3.36</v>
       </c>
-      <c r="AC13" s="15">
+      <c r="AC13" s="10">
         <v>3.01</v>
       </c>
-      <c r="AD13" s="15">
+      <c r="AD13" s="10">
         <v>4.45</v>
       </c>
-      <c r="AE13" s="15">
+      <c r="AE13" s="10">
         <v>3.03</v>
       </c>
-      <c r="AF13" s="15">
+      <c r="AF13" s="10">
         <v>2.88</v>
       </c>
-      <c r="AG13" s="15">
+      <c r="AG13" s="10">
         <v>3.56</v>
       </c>
-      <c r="AH13" s="15">
+      <c r="AH13" s="10">
         <v>3.36</v>
       </c>
-      <c r="AI13" s="15">
+      <c r="AI13" s="10">
         <v>3.14</v>
       </c>
-      <c r="AJ13" s="15">
+      <c r="AJ13" s="10">
         <v>4.1900000000000004</v>
       </c>
-      <c r="AK13" s="15">
+      <c r="AK13" s="10">
         <v>3.92</v>
       </c>
-      <c r="AL13" s="15">
+      <c r="AL13" s="10">
         <v>3.84</v>
       </c>
-      <c r="AM13" s="15">
+      <c r="AM13" s="10">
         <v>4.17</v>
       </c>
-      <c r="AN13" s="15">
+      <c r="AN13" s="10">
         <v>3.79</v>
       </c>
-      <c r="AO13" s="15">
+      <c r="AO13" s="10">
         <v>3.49</v>
       </c>
-      <c r="AP13" s="15">
+      <c r="AP13" s="10">
         <v>4.8899999999999997</v>
       </c>
-      <c r="AQ13" s="15">
+      <c r="AQ13" s="10">
         <v>4.76</v>
       </c>
-      <c r="AR13" s="15">
+      <c r="AR13" s="10">
         <v>4.75</v>
       </c>
-      <c r="AS13" s="15">
+      <c r="AS13" s="10">
         <v>4.78</v>
       </c>
     </row>
-    <row r="14" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20" t="s">
+    <row r="14" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="10">
         <v>4.08</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="10">
         <v>2.81</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="10">
         <v>6.73</v>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="10">
         <v>3.32</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="10">
         <v>2.31</v>
       </c>
-      <c r="I14" s="15">
+      <c r="I14" s="10">
         <v>5.54</v>
       </c>
-      <c r="J14" s="15">
+      <c r="J14" s="10">
         <v>2.91</v>
       </c>
-      <c r="K14" s="15">
+      <c r="K14" s="10">
         <v>2.36</v>
       </c>
-      <c r="L14" s="15">
+      <c r="L14" s="10">
         <v>4.2</v>
       </c>
-      <c r="M14" s="15">
+      <c r="M14" s="10">
         <v>3.06</v>
       </c>
-      <c r="N14" s="15">
+      <c r="N14" s="10">
         <v>2.62</v>
       </c>
-      <c r="O14" s="15">
+      <c r="O14" s="10">
         <v>4.08</v>
       </c>
-      <c r="P14" s="15">
+      <c r="P14" s="10">
         <v>3.43</v>
       </c>
-      <c r="Q14" s="15">
+      <c r="Q14" s="10">
         <v>2.64</v>
       </c>
-      <c r="R14" s="15">
+      <c r="R14" s="10">
         <v>5.34</v>
       </c>
-      <c r="S14" s="15">
+      <c r="S14" s="10">
         <v>3.59</v>
       </c>
-      <c r="T14" s="15">
+      <c r="T14" s="10">
         <v>2.9</v>
       </c>
-      <c r="U14" s="15">
+      <c r="U14" s="10">
         <v>5.24</v>
       </c>
-      <c r="V14" s="15">
+      <c r="V14" s="10">
         <v>3.68</v>
       </c>
-      <c r="W14" s="15">
+      <c r="W14" s="10">
         <v>3.02</v>
       </c>
-      <c r="X14" s="15">
+      <c r="X14" s="10">
         <v>5.24</v>
       </c>
-      <c r="Y14" s="15">
+      <c r="Y14" s="10">
         <v>4.03</v>
       </c>
-      <c r="Z14" s="15">
+      <c r="Z14" s="10">
         <v>3.22</v>
       </c>
-      <c r="AA14" s="15">
+      <c r="AA14" s="10">
         <v>5.87</v>
       </c>
-      <c r="AB14" s="15">
+      <c r="AB14" s="10">
         <v>4.5199999999999996</v>
       </c>
-      <c r="AC14" s="15">
+      <c r="AC14" s="10">
         <v>4</v>
       </c>
-      <c r="AD14" s="15">
+      <c r="AD14" s="10">
         <v>5.94</v>
       </c>
-      <c r="AE14" s="15">
+      <c r="AE14" s="10">
         <v>4.33</v>
       </c>
-      <c r="AF14" s="15">
+      <c r="AF14" s="10">
         <v>3.79</v>
       </c>
-      <c r="AG14" s="15">
+      <c r="AG14" s="10">
         <v>6.16</v>
       </c>
-      <c r="AH14" s="15">
+      <c r="AH14" s="10">
         <v>4.8600000000000003</v>
       </c>
-      <c r="AI14" s="15">
+      <c r="AI14" s="10">
         <v>4.53</v>
       </c>
-      <c r="AJ14" s="15">
+      <c r="AJ14" s="10">
         <v>5.97</v>
       </c>
-      <c r="AK14" s="15">
+      <c r="AK14" s="10">
         <v>4.95</v>
       </c>
-      <c r="AL14" s="15">
+      <c r="AL14" s="10">
         <v>4.63</v>
       </c>
-      <c r="AM14" s="15">
+      <c r="AM14" s="10">
         <v>5.89</v>
       </c>
-      <c r="AN14" s="15">
+      <c r="AN14" s="10">
         <v>4.62</v>
       </c>
-      <c r="AO14" s="15">
+      <c r="AO14" s="10">
         <v>4.07</v>
       </c>
-      <c r="AP14" s="15">
+      <c r="AP14" s="10">
         <v>6.49</v>
       </c>
-      <c r="AQ14" s="15">
+      <c r="AQ14" s="10">
         <v>5.0999999999999996</v>
       </c>
-      <c r="AR14" s="15">
+      <c r="AR14" s="10">
         <v>4.5999999999999996</v>
       </c>
-      <c r="AS14" s="15">
+      <c r="AS14" s="10">
         <v>6.84</v>
       </c>
     </row>
-    <row r="15" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="20" t="s">
+    <row r="15" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="10">
         <v>2.92</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="10">
         <v>1.84</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="10">
         <v>4.96</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="10">
         <v>2.6</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="10">
         <v>1.61</v>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="10">
         <v>4.42</v>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="10">
         <v>2.11</v>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="10">
         <v>1.54</v>
       </c>
-      <c r="L15" s="15">
+      <c r="L15" s="10">
         <v>3.26</v>
       </c>
-      <c r="M15" s="15">
+      <c r="M15" s="10">
         <v>2.11</v>
       </c>
-      <c r="N15" s="15">
+      <c r="N15" s="10">
         <v>1.5</v>
       </c>
-      <c r="O15" s="15">
+      <c r="O15" s="10">
         <v>3.43</v>
       </c>
-      <c r="P15" s="15">
+      <c r="P15" s="10">
         <v>2.7</v>
       </c>
-      <c r="Q15" s="15">
+      <c r="Q15" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R15" s="15">
+      <c r="R15" s="10">
         <v>3.64</v>
       </c>
-      <c r="S15" s="15">
+      <c r="S15" s="10">
         <v>2.44</v>
       </c>
-      <c r="T15" s="15">
+      <c r="T15" s="10">
         <v>1.78</v>
       </c>
-      <c r="U15" s="15">
+      <c r="U15" s="10">
         <v>3.98</v>
       </c>
-      <c r="V15" s="15">
+      <c r="V15" s="10">
         <v>2.5499999999999998</v>
       </c>
-      <c r="W15" s="15">
+      <c r="W15" s="10">
         <v>1.7</v>
       </c>
-      <c r="X15" s="15">
+      <c r="X15" s="10">
         <v>4.4800000000000004</v>
       </c>
-      <c r="Y15" s="15">
+      <c r="Y15" s="10">
         <v>2.92</v>
       </c>
-      <c r="Z15" s="15">
+      <c r="Z15" s="10">
         <v>2.16</v>
       </c>
-      <c r="AA15" s="15">
+      <c r="AA15" s="10">
         <v>4.75</v>
       </c>
-      <c r="AB15" s="15">
+      <c r="AB15" s="10">
         <v>3.32</v>
       </c>
-      <c r="AC15" s="15">
+      <c r="AC15" s="10">
         <v>2.44</v>
       </c>
-      <c r="AD15" s="15">
+      <c r="AD15" s="10">
         <v>6</v>
       </c>
-      <c r="AE15" s="15">
+      <c r="AE15" s="10">
         <v>3.52</v>
       </c>
-      <c r="AF15" s="15">
+      <c r="AF15" s="10">
         <v>3.06</v>
       </c>
-      <c r="AG15" s="15">
+      <c r="AG15" s="10">
         <v>5.1100000000000003</v>
       </c>
-      <c r="AH15" s="15">
+      <c r="AH15" s="10">
         <v>3.68</v>
       </c>
-      <c r="AI15" s="15">
+      <c r="AI15" s="10">
         <v>3.23</v>
       </c>
-      <c r="AJ15" s="15">
+      <c r="AJ15" s="10">
         <v>5.41</v>
       </c>
-      <c r="AK15" s="15">
+      <c r="AK15" s="10">
         <v>3.94</v>
       </c>
-      <c r="AL15" s="15">
+      <c r="AL15" s="10">
         <v>3.48</v>
       </c>
-      <c r="AM15" s="15">
+      <c r="AM15" s="10">
         <v>5.71</v>
       </c>
-      <c r="AN15" s="15">
+      <c r="AN15" s="10">
         <v>3.69</v>
       </c>
-      <c r="AO15" s="15">
+      <c r="AO15" s="10">
         <v>3.2</v>
       </c>
-      <c r="AP15" s="15">
+      <c r="AP15" s="10">
         <v>6.02</v>
       </c>
-      <c r="AQ15" s="15">
+      <c r="AQ15" s="10">
         <v>3.78</v>
       </c>
-      <c r="AR15" s="15">
+      <c r="AR15" s="10">
         <v>3.25</v>
       </c>
-      <c r="AS15" s="15">
+      <c r="AS15" s="10">
         <v>6.33</v>
       </c>
     </row>
-    <row r="16" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
-      <c r="B16" s="20" t="s">
+    <row r="16" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="10">
         <v>2.1</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="10">
         <v>1.28</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="10">
         <v>4.0599999999999996</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="10">
         <v>1.89</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="10">
         <v>1.35</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="10">
         <v>3.31</v>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="10">
         <v>1.84</v>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="10">
         <v>1.4</v>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="10">
         <v>3.15</v>
       </c>
-      <c r="M16" s="15">
+      <c r="M16" s="10">
         <v>1.78</v>
       </c>
-      <c r="N16" s="15">
+      <c r="N16" s="10">
         <v>1.28</v>
       </c>
-      <c r="O16" s="15">
+      <c r="O16" s="10">
         <v>3.41</v>
       </c>
-      <c r="P16" s="15">
+      <c r="P16" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="Q16" s="15">
+      <c r="Q16" s="10">
         <v>1.73</v>
       </c>
-      <c r="R16" s="15">
+      <c r="R16" s="10">
         <v>3.85</v>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="10">
         <v>1.84</v>
       </c>
-      <c r="T16" s="15">
+      <c r="T16" s="10">
         <v>1.5</v>
       </c>
-      <c r="U16" s="15">
+      <c r="U16" s="10">
         <v>3.32</v>
       </c>
-      <c r="V16" s="15">
+      <c r="V16" s="10">
         <v>2.08</v>
       </c>
-      <c r="W16" s="15">
+      <c r="W16" s="10">
         <v>1.8</v>
       </c>
-      <c r="X16" s="15">
+      <c r="X16" s="10">
         <v>3.36</v>
       </c>
-      <c r="Y16" s="15">
+      <c r="Y16" s="10">
         <v>2.59</v>
       </c>
-      <c r="Z16" s="15">
+      <c r="Z16" s="10">
         <v>2.13</v>
       </c>
-      <c r="AA16" s="15">
+      <c r="AA16" s="10">
         <v>4.82</v>
       </c>
-      <c r="AB16" s="15">
+      <c r="AB16" s="10">
         <v>2.46</v>
       </c>
-      <c r="AC16" s="15">
+      <c r="AC16" s="10">
         <v>2.16</v>
       </c>
-      <c r="AD16" s="15">
+      <c r="AD16" s="10">
         <v>4.13</v>
       </c>
-      <c r="AE16" s="15">
+      <c r="AE16" s="10">
         <v>3.27</v>
       </c>
-      <c r="AF16" s="15">
+      <c r="AF16" s="10">
         <v>2.91</v>
       </c>
-      <c r="AG16" s="15">
+      <c r="AG16" s="10">
         <v>5.45</v>
       </c>
-      <c r="AH16" s="15">
+      <c r="AH16" s="10">
         <v>3.39</v>
       </c>
-      <c r="AI16" s="15">
+      <c r="AI16" s="10">
         <v>3</v>
       </c>
-      <c r="AJ16" s="15">
+      <c r="AJ16" s="10">
         <v>5.71</v>
       </c>
-      <c r="AK16" s="15">
+      <c r="AK16" s="10">
         <v>3.36</v>
       </c>
-      <c r="AL16" s="15">
+      <c r="AL16" s="10">
         <v>2.99</v>
       </c>
-      <c r="AM16" s="15">
+      <c r="AM16" s="10">
         <v>5.5</v>
       </c>
-      <c r="AN16" s="15">
+      <c r="AN16" s="10">
         <v>3.64</v>
       </c>
-      <c r="AO16" s="15">
+      <c r="AO16" s="10">
         <v>3.13</v>
       </c>
-      <c r="AP16" s="15">
+      <c r="AP16" s="10">
         <v>6.82</v>
       </c>
-      <c r="AQ16" s="15">
+      <c r="AQ16" s="10">
         <v>4.2</v>
       </c>
-      <c r="AR16" s="15">
+      <c r="AR16" s="10">
         <v>3.69</v>
       </c>
-      <c r="AS16" s="15">
+      <c r="AS16" s="10">
         <v>7.42</v>
       </c>
     </row>
-    <row r="17" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
-      <c r="B17" s="20" t="s">
+    <row r="17" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="10">
         <v>1.68</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="10">
         <v>1.49</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="10">
         <v>2.64</v>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="10">
         <v>1.57</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="10">
         <v>1.31</v>
       </c>
-      <c r="I17" s="15">
+      <c r="I17" s="10">
         <v>2.81</v>
       </c>
-      <c r="J17" s="15">
+      <c r="J17" s="10">
         <v>1.49</v>
       </c>
-      <c r="K17" s="15">
+      <c r="K17" s="10">
         <v>1.33</v>
       </c>
-      <c r="L17" s="15">
+      <c r="L17" s="10">
         <v>2.35</v>
       </c>
-      <c r="M17" s="15">
+      <c r="M17" s="10">
         <v>1.87</v>
       </c>
-      <c r="N17" s="15">
+      <c r="N17" s="10">
         <v>1.7</v>
       </c>
-      <c r="O17" s="15">
+      <c r="O17" s="10">
         <v>2.76</v>
       </c>
-      <c r="P17" s="15">
+      <c r="P17" s="10">
         <v>1.84</v>
       </c>
-      <c r="Q17" s="15">
+      <c r="Q17" s="10">
         <v>1.61</v>
       </c>
-      <c r="R17" s="15">
+      <c r="R17" s="10">
         <v>3.1</v>
       </c>
-      <c r="S17" s="15">
+      <c r="S17" s="10">
         <v>1.75</v>
       </c>
-      <c r="T17" s="15">
+      <c r="T17" s="10">
         <v>1.53</v>
       </c>
-      <c r="U17" s="15">
+      <c r="U17" s="10">
         <v>2.96</v>
       </c>
-      <c r="V17" s="15">
+      <c r="V17" s="10">
         <v>1.97</v>
       </c>
-      <c r="W17" s="15">
+      <c r="W17" s="10">
         <v>1.86</v>
       </c>
-      <c r="X17" s="15">
+      <c r="X17" s="10">
         <v>2.6</v>
       </c>
-      <c r="Y17" s="15">
+      <c r="Y17" s="10">
         <v>2.37</v>
       </c>
-      <c r="Z17" s="15">
+      <c r="Z17" s="10">
         <v>2.09</v>
       </c>
-      <c r="AA17" s="15">
+      <c r="AA17" s="10">
         <v>3.92</v>
       </c>
-      <c r="AB17" s="15">
+      <c r="AB17" s="10">
         <v>2.46</v>
       </c>
-      <c r="AC17" s="15">
+      <c r="AC17" s="10">
         <v>2.15</v>
       </c>
-      <c r="AD17" s="15">
+      <c r="AD17" s="10">
         <v>4.3099999999999996</v>
       </c>
-      <c r="AE17" s="15">
+      <c r="AE17" s="10">
         <v>2.61</v>
       </c>
-      <c r="AF17" s="15">
+      <c r="AF17" s="10">
         <v>2.2400000000000002</v>
       </c>
-      <c r="AG17" s="15">
+      <c r="AG17" s="10">
         <v>4.88</v>
       </c>
-      <c r="AH17" s="15">
+      <c r="AH17" s="10">
         <v>3.07</v>
       </c>
-      <c r="AI17" s="15">
+      <c r="AI17" s="10">
         <v>2.72</v>
       </c>
-      <c r="AJ17" s="15">
+      <c r="AJ17" s="10">
         <v>5.32</v>
       </c>
-      <c r="AK17" s="15">
+      <c r="AK17" s="10">
         <v>3.19</v>
       </c>
-      <c r="AL17" s="15">
+      <c r="AL17" s="10">
         <v>2.79</v>
       </c>
-      <c r="AM17" s="15">
+      <c r="AM17" s="10">
         <v>5.66</v>
       </c>
-      <c r="AN17" s="15">
+      <c r="AN17" s="10">
         <v>3.22</v>
       </c>
-      <c r="AO17" s="15">
+      <c r="AO17" s="10">
         <v>2.72</v>
       </c>
-      <c r="AP17" s="15">
+      <c r="AP17" s="10">
         <v>6.36</v>
       </c>
-      <c r="AQ17" s="15">
+      <c r="AQ17" s="10">
         <v>3.56</v>
       </c>
-      <c r="AR17" s="15">
+      <c r="AR17" s="10">
         <v>2.92</v>
       </c>
-      <c r="AS17" s="15">
+      <c r="AS17" s="10">
         <v>7.84</v>
       </c>
     </row>
-    <row r="18" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="20" t="s">
+    <row r="18" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="10">
         <v>2.84</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="10">
         <v>2.02</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="10">
         <v>4.8499999999999996</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="10">
         <v>2.54</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="10">
         <v>1.87</v>
       </c>
-      <c r="I18" s="15">
+      <c r="I18" s="10">
         <v>4.26</v>
       </c>
-      <c r="J18" s="15">
+      <c r="J18" s="10">
         <v>2.2599999999999998</v>
       </c>
-      <c r="K18" s="15">
+      <c r="K18" s="10">
         <v>1.81</v>
       </c>
-      <c r="L18" s="15">
+      <c r="L18" s="10">
         <v>3.52</v>
       </c>
-      <c r="M18" s="15">
+      <c r="M18" s="10">
         <v>2.31</v>
       </c>
-      <c r="N18" s="15">
+      <c r="N18" s="10">
         <v>1.9</v>
       </c>
-      <c r="O18" s="15">
+      <c r="O18" s="10">
         <v>3.49</v>
       </c>
-      <c r="P18" s="15">
+      <c r="P18" s="10">
         <v>2.66</v>
       </c>
-      <c r="Q18" s="15">
+      <c r="Q18" s="10">
         <v>2.1800000000000002</v>
       </c>
-      <c r="R18" s="15">
+      <c r="R18" s="10">
         <v>4.1399999999999997</v>
       </c>
-      <c r="S18" s="15">
+      <c r="S18" s="10">
         <v>2.48</v>
       </c>
-      <c r="T18" s="15">
+      <c r="T18" s="10">
         <v>1.96</v>
       </c>
-      <c r="U18" s="15">
+      <c r="U18" s="10">
         <v>4.16</v>
       </c>
-      <c r="V18" s="15">
+      <c r="V18" s="10">
         <v>2.62</v>
       </c>
-      <c r="W18" s="15">
+      <c r="W18" s="10">
         <v>2.17</v>
       </c>
-      <c r="X18" s="15">
+      <c r="X18" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="Y18" s="15">
+      <c r="Y18" s="10">
         <v>2.96</v>
       </c>
-      <c r="Z18" s="15">
+      <c r="Z18" s="10">
         <v>2.36</v>
       </c>
-      <c r="AA18" s="15">
+      <c r="AA18" s="10">
         <v>4.93</v>
       </c>
-      <c r="AB18" s="15">
+      <c r="AB18" s="10">
         <v>3.15</v>
       </c>
-      <c r="AC18" s="15">
+      <c r="AC18" s="10">
         <v>2.65</v>
       </c>
-      <c r="AD18" s="15">
+      <c r="AD18" s="10">
         <v>5.07</v>
       </c>
-      <c r="AE18" s="15">
+      <c r="AE18" s="10">
         <v>3.33</v>
       </c>
-      <c r="AF18" s="15">
+      <c r="AF18" s="10">
         <v>2.93</v>
       </c>
-      <c r="AG18" s="15">
+      <c r="AG18" s="10">
         <v>5.07</v>
       </c>
-      <c r="AH18" s="15">
+      <c r="AH18" s="10">
         <v>3.64</v>
       </c>
-      <c r="AI18" s="15">
+      <c r="AI18" s="10">
         <v>3.26</v>
       </c>
-      <c r="AJ18" s="15">
+      <c r="AJ18" s="10">
         <v>5.34</v>
       </c>
-      <c r="AK18" s="15">
+      <c r="AK18" s="10">
         <v>3.81</v>
       </c>
-      <c r="AL18" s="15">
+      <c r="AL18" s="10">
         <v>3.44</v>
       </c>
-      <c r="AM18" s="15">
+      <c r="AM18" s="10">
         <v>5.38</v>
       </c>
-      <c r="AN18" s="15">
+      <c r="AN18" s="10">
         <v>3.76</v>
       </c>
-      <c r="AO18" s="15">
+      <c r="AO18" s="10">
         <v>3.27</v>
       </c>
-      <c r="AP18" s="15">
+      <c r="AP18" s="10">
         <v>6.11</v>
       </c>
-      <c r="AQ18" s="15">
+      <c r="AQ18" s="10">
         <v>4.2300000000000004</v>
       </c>
-      <c r="AR18" s="15">
+      <c r="AR18" s="10">
         <v>3.76</v>
       </c>
-      <c r="AS18" s="15">
+      <c r="AS18" s="10">
         <v>6.55</v>
       </c>
     </row>
-    <row r="19" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="20" t="s">
+    <row r="19" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="10">
         <v>4.21</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="10">
         <v>3.52</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="10">
         <v>5.35</v>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="10">
         <v>3.85</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="10">
         <v>3.38</v>
       </c>
-      <c r="I19" s="15">
+      <c r="I19" s="10">
         <v>4.7</v>
       </c>
-      <c r="J19" s="15">
+      <c r="J19" s="10">
         <v>3.57</v>
       </c>
-      <c r="K19" s="15">
+      <c r="K19" s="10">
         <v>3.01</v>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="10">
         <v>4.68</v>
       </c>
-      <c r="M19" s="15">
+      <c r="M19" s="10">
         <v>3.37</v>
       </c>
-      <c r="N19" s="15">
+      <c r="N19" s="10">
         <v>2.87</v>
       </c>
-      <c r="O19" s="15">
+      <c r="O19" s="10">
         <v>4.45</v>
       </c>
-      <c r="P19" s="15">
+      <c r="P19" s="10">
         <v>4.04</v>
       </c>
-      <c r="Q19" s="15">
+      <c r="Q19" s="10">
         <v>3.36</v>
       </c>
-      <c r="R19" s="15">
+      <c r="R19" s="10">
         <v>5.57</v>
       </c>
-      <c r="S19" s="15">
+      <c r="S19" s="10">
         <v>3.55</v>
       </c>
-      <c r="T19" s="15">
+      <c r="T19" s="10">
         <v>2.86</v>
       </c>
-      <c r="U19" s="15">
+      <c r="U19" s="10">
         <v>5.24</v>
       </c>
-      <c r="V19" s="15">
+      <c r="V19" s="10">
         <v>3.48</v>
       </c>
-      <c r="W19" s="15">
+      <c r="W19" s="10">
         <v>2.84</v>
       </c>
-      <c r="X19" s="15">
+      <c r="X19" s="10">
         <v>5.09</v>
       </c>
-      <c r="Y19" s="15">
+      <c r="Y19" s="10">
         <v>3.69</v>
       </c>
-      <c r="Z19" s="15">
+      <c r="Z19" s="10">
         <v>2.94</v>
       </c>
-      <c r="AA19" s="15">
+      <c r="AA19" s="10">
         <v>5.46</v>
       </c>
-      <c r="AB19" s="15">
+      <c r="AB19" s="10">
         <v>4.1100000000000003</v>
       </c>
-      <c r="AC19" s="15">
+      <c r="AC19" s="10">
         <v>3.58</v>
       </c>
-      <c r="AD19" s="15">
+      <c r="AD19" s="10">
         <v>5.61</v>
       </c>
-      <c r="AE19" s="15">
+      <c r="AE19" s="10">
         <v>3.38</v>
       </c>
-      <c r="AF19" s="15">
+      <c r="AF19" s="10">
         <v>3.27</v>
       </c>
-      <c r="AG19" s="15">
+      <c r="AG19" s="10">
         <v>3.72</v>
       </c>
-      <c r="AH19" s="15">
+      <c r="AH19" s="10">
         <v>3.98</v>
       </c>
-      <c r="AI19" s="15">
+      <c r="AI19" s="10">
         <v>3.97</v>
       </c>
-      <c r="AJ19" s="15">
+      <c r="AJ19" s="10">
         <v>4.04</v>
       </c>
-      <c r="AK19" s="15">
+      <c r="AK19" s="10">
         <v>4.29</v>
       </c>
-      <c r="AL19" s="15">
+      <c r="AL19" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AM19" s="15">
+      <c r="AM19" s="10">
         <v>4.92</v>
       </c>
-      <c r="AN19" s="15">
+      <c r="AN19" s="10">
         <v>4.03</v>
       </c>
-      <c r="AO19" s="15">
+      <c r="AO19" s="10">
         <v>3.75</v>
       </c>
-      <c r="AP19" s="15">
+      <c r="AP19" s="10">
         <v>5.04</v>
       </c>
-      <c r="AQ19" s="15">
+      <c r="AQ19" s="10">
         <v>5.25</v>
       </c>
-      <c r="AR19" s="15">
+      <c r="AR19" s="10">
         <v>5.08</v>
       </c>
-      <c r="AS19" s="15">
+      <c r="AS19" s="10">
         <v>5.85</v>
       </c>
     </row>
-    <row r="20" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20" t="s">
+    <row r="20" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="10">
         <v>4.75</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="10">
         <v>3.34</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="10">
         <v>7.56</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="10">
         <v>3.71</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="10">
         <v>2.42</v>
       </c>
-      <c r="I20" s="15">
+      <c r="I20" s="10">
         <v>6.44</v>
       </c>
-      <c r="J20" s="15">
+      <c r="J20" s="10">
         <v>3.66</v>
       </c>
-      <c r="K20" s="15">
+      <c r="K20" s="10">
         <v>2.9</v>
       </c>
-      <c r="L20" s="15">
+      <c r="L20" s="10">
         <v>5.4</v>
       </c>
-      <c r="M20" s="15">
+      <c r="M20" s="10">
         <v>3.41</v>
       </c>
-      <c r="N20" s="15">
+      <c r="N20" s="10">
         <v>2.9</v>
       </c>
-      <c r="O20" s="15">
+      <c r="O20" s="10">
         <v>4.55</v>
       </c>
-      <c r="P20" s="15">
+      <c r="P20" s="10">
         <v>4.32</v>
       </c>
-      <c r="Q20" s="15">
+      <c r="Q20" s="10">
         <v>3.33</v>
       </c>
-      <c r="R20" s="15">
+      <c r="R20" s="10">
         <v>6.56</v>
       </c>
-      <c r="S20" s="15">
+      <c r="S20" s="10">
         <v>4.6399999999999997</v>
       </c>
-      <c r="T20" s="15">
+      <c r="T20" s="10">
         <v>3.6</v>
       </c>
-      <c r="U20" s="15">
+      <c r="U20" s="10">
         <v>6.96</v>
       </c>
-      <c r="V20" s="15">
+      <c r="V20" s="10">
         <v>4.32</v>
       </c>
-      <c r="W20" s="15">
+      <c r="W20" s="10">
         <v>3.49</v>
       </c>
-      <c r="X20" s="15">
+      <c r="X20" s="10">
         <v>6.22</v>
       </c>
-      <c r="Y20" s="15">
+      <c r="Y20" s="10">
         <v>4.8899999999999997</v>
       </c>
-      <c r="Z20" s="15">
+      <c r="Z20" s="10">
         <v>3.64</v>
       </c>
-      <c r="AA20" s="15">
+      <c r="AA20" s="10">
         <v>7.53</v>
       </c>
-      <c r="AB20" s="15">
+      <c r="AB20" s="10">
         <v>5.37</v>
       </c>
-      <c r="AC20" s="15">
+      <c r="AC20" s="10">
         <v>4.5199999999999996</v>
       </c>
-      <c r="AD20" s="15">
+      <c r="AD20" s="10">
         <v>7.57</v>
       </c>
-      <c r="AE20" s="15">
+      <c r="AE20" s="10">
         <v>5.26</v>
       </c>
-      <c r="AF20" s="15">
+      <c r="AF20" s="10">
         <v>4.91</v>
       </c>
-      <c r="AG20" s="15">
+      <c r="AG20" s="10">
         <v>6.44</v>
       </c>
-      <c r="AH20" s="15">
+      <c r="AH20" s="10">
         <v>5.71</v>
       </c>
-      <c r="AI20" s="15">
+      <c r="AI20" s="10">
         <v>5.38</v>
       </c>
-      <c r="AJ20" s="15">
+      <c r="AJ20" s="10">
         <v>6.78</v>
       </c>
-      <c r="AK20" s="15">
+      <c r="AK20" s="10">
         <v>6.14</v>
       </c>
-      <c r="AL20" s="15">
+      <c r="AL20" s="10">
         <v>5.68</v>
       </c>
-      <c r="AM20" s="15">
+      <c r="AM20" s="10">
         <v>7.53</v>
       </c>
-      <c r="AN20" s="15">
+      <c r="AN20" s="10">
         <v>5.43</v>
       </c>
-      <c r="AO20" s="15">
+      <c r="AO20" s="10">
         <v>4.71</v>
       </c>
-      <c r="AP20" s="15">
+      <c r="AP20" s="10">
         <v>7.91</v>
       </c>
-      <c r="AQ20" s="15">
+      <c r="AQ20" s="10">
         <v>5.37</v>
       </c>
-      <c r="AR20" s="15">
+      <c r="AR20" s="10">
         <v>4.45</v>
       </c>
-      <c r="AS20" s="15">
+      <c r="AS20" s="10">
         <v>8.4700000000000006</v>
       </c>
     </row>
-    <row r="21" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
-      <c r="B21" s="20" t="s">
+    <row r="21" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="10">
         <v>3.34</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="10">
         <v>1.85</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="10">
         <v>6.08</v>
       </c>
-      <c r="G21" s="15">
+      <c r="G21" s="10">
         <v>2.69</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="10">
         <v>1.82</v>
       </c>
-      <c r="I21" s="15">
+      <c r="I21" s="10">
         <v>4.3</v>
       </c>
-      <c r="J21" s="15">
+      <c r="J21" s="10">
         <v>2.31</v>
       </c>
-      <c r="K21" s="15">
+      <c r="K21" s="10">
         <v>1.75</v>
       </c>
-      <c r="L21" s="15">
+      <c r="L21" s="10">
         <v>3.41</v>
       </c>
-      <c r="M21" s="15">
+      <c r="M21" s="10">
         <v>2.58</v>
       </c>
-      <c r="N21" s="15">
+      <c r="N21" s="10">
         <v>1.7</v>
       </c>
-      <c r="O21" s="15">
+      <c r="O21" s="10">
         <v>4.46</v>
       </c>
-      <c r="P21" s="15">
+      <c r="P21" s="10">
         <v>2.93</v>
       </c>
-      <c r="Q21" s="15">
+      <c r="Q21" s="10">
         <v>2.37</v>
       </c>
-      <c r="R21" s="15">
+      <c r="R21" s="10">
         <v>4.24</v>
       </c>
-      <c r="S21" s="15">
+      <c r="S21" s="10">
         <v>2.85</v>
       </c>
-      <c r="T21" s="15">
+      <c r="T21" s="10">
         <v>2.04</v>
       </c>
-      <c r="U21" s="15">
+      <c r="U21" s="10">
         <v>4.63</v>
       </c>
-      <c r="V21" s="15">
+      <c r="V21" s="10">
         <v>3.19</v>
       </c>
-      <c r="W21" s="15">
+      <c r="W21" s="10">
         <v>2.1</v>
       </c>
-      <c r="X21" s="15">
+      <c r="X21" s="10">
         <v>5.47</v>
       </c>
-      <c r="Y21" s="15">
+      <c r="Y21" s="10">
         <v>3.07</v>
       </c>
-      <c r="Z21" s="15">
+      <c r="Z21" s="10">
         <v>2.21</v>
       </c>
-      <c r="AA21" s="15">
+      <c r="AA21" s="10">
         <v>5.09</v>
       </c>
-      <c r="AB21" s="15">
+      <c r="AB21" s="10">
         <v>4.12</v>
       </c>
-      <c r="AC21" s="15">
+      <c r="AC21" s="10">
         <v>2.88</v>
       </c>
-      <c r="AD21" s="15">
+      <c r="AD21" s="10">
         <v>7.82</v>
       </c>
-      <c r="AE21" s="15">
+      <c r="AE21" s="10">
         <v>3.9</v>
       </c>
-      <c r="AF21" s="15">
+      <c r="AF21" s="10">
         <v>3.41</v>
       </c>
-      <c r="AG21" s="15">
+      <c r="AG21" s="10">
         <v>5.56</v>
       </c>
-      <c r="AH21" s="15">
+      <c r="AH21" s="10">
         <v>4.25</v>
       </c>
-      <c r="AI21" s="15">
+      <c r="AI21" s="10">
         <v>3.69</v>
       </c>
-      <c r="AJ21" s="15">
+      <c r="AJ21" s="10">
         <v>6.5</v>
       </c>
-      <c r="AK21" s="15">
+      <c r="AK21" s="10">
         <v>4.5199999999999996</v>
       </c>
-      <c r="AL21" s="15">
+      <c r="AL21" s="10">
         <v>3.87</v>
       </c>
-      <c r="AM21" s="15">
+      <c r="AM21" s="10">
         <v>6.97</v>
       </c>
-      <c r="AN21" s="15">
+      <c r="AN21" s="10">
         <v>4.25</v>
       </c>
-      <c r="AO21" s="15">
+      <c r="AO21" s="10">
         <v>3.41</v>
       </c>
-      <c r="AP21" s="15">
+      <c r="AP21" s="10">
         <v>8.32</v>
       </c>
-      <c r="AQ21" s="15">
+      <c r="AQ21" s="10">
         <v>3.81</v>
       </c>
-      <c r="AR21" s="15">
+      <c r="AR21" s="10">
         <v>3.23</v>
       </c>
-      <c r="AS21" s="15">
+      <c r="AS21" s="10">
         <v>6.8</v>
       </c>
     </row>
-    <row r="22" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="20" t="s">
+    <row r="22" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14"/>
+      <c r="B22" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="10">
         <v>2.4300000000000002</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="10">
         <v>1.62</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="G22" s="15">
+      <c r="G22" s="10">
         <v>2</v>
       </c>
-      <c r="H22" s="15">
+      <c r="H22" s="10">
         <v>1.67</v>
       </c>
-      <c r="I22" s="15">
+      <c r="I22" s="10">
         <v>2.87</v>
       </c>
-      <c r="J22" s="15">
+      <c r="J22" s="10">
         <v>2</v>
       </c>
-      <c r="K22" s="15">
+      <c r="K22" s="10">
         <v>1.36</v>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="10">
         <v>3.94</v>
       </c>
-      <c r="M22" s="15">
+      <c r="M22" s="10">
         <v>2.09</v>
       </c>
-      <c r="N22" s="15">
+      <c r="N22" s="10">
         <v>1.5</v>
       </c>
-      <c r="O22" s="15">
+      <c r="O22" s="10">
         <v>4</v>
       </c>
-      <c r="P22" s="15">
+      <c r="P22" s="10">
         <v>2.5299999999999998</v>
       </c>
-      <c r="Q22" s="15">
+      <c r="Q22" s="10">
         <v>1.99</v>
       </c>
-      <c r="R22" s="15">
+      <c r="R22" s="10">
         <v>4.4400000000000004</v>
       </c>
-      <c r="S22" s="15">
+      <c r="S22" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="T22" s="15">
+      <c r="T22" s="10">
         <v>1.97</v>
       </c>
-      <c r="U22" s="15">
+      <c r="U22" s="10">
         <v>3.78</v>
       </c>
-      <c r="V22" s="15">
+      <c r="V22" s="10">
         <v>2.31</v>
       </c>
-      <c r="W22" s="15">
+      <c r="W22" s="10">
         <v>2.08</v>
       </c>
-      <c r="X22" s="15">
+      <c r="X22" s="10">
         <v>3.39</v>
       </c>
-      <c r="Y22" s="15">
+      <c r="Y22" s="10">
         <v>3.09</v>
       </c>
-      <c r="Z22" s="15">
+      <c r="Z22" s="10">
         <v>2.5499999999999998</v>
       </c>
-      <c r="AA22" s="15">
+      <c r="AA22" s="10">
         <v>5.56</v>
       </c>
-      <c r="AB22" s="15">
+      <c r="AB22" s="10">
         <v>2.89</v>
       </c>
-      <c r="AC22" s="15">
+      <c r="AC22" s="10">
         <v>2.42</v>
       </c>
-      <c r="AD22" s="15">
+      <c r="AD22" s="10">
         <v>5.49</v>
       </c>
-      <c r="AE22" s="15">
+      <c r="AE22" s="10">
         <v>3.51</v>
       </c>
-      <c r="AF22" s="15">
+      <c r="AF22" s="10">
         <v>3.03</v>
       </c>
-      <c r="AG22" s="15">
+      <c r="AG22" s="10">
         <v>6.3</v>
       </c>
-      <c r="AH22" s="15">
+      <c r="AH22" s="10">
         <v>3.77</v>
       </c>
-      <c r="AI22" s="15">
+      <c r="AI22" s="10">
         <v>3.26</v>
       </c>
-      <c r="AJ22" s="15">
+      <c r="AJ22" s="10">
         <v>6.71</v>
       </c>
-      <c r="AK22" s="15">
+      <c r="AK22" s="10">
         <v>3.54</v>
       </c>
-      <c r="AL22" s="15">
+      <c r="AL22" s="10">
         <v>3.04</v>
       </c>
-      <c r="AM22" s="15">
+      <c r="AM22" s="10">
         <v>6.47</v>
       </c>
-      <c r="AN22" s="15">
+      <c r="AN22" s="10">
         <v>3.91</v>
       </c>
-      <c r="AO22" s="15">
+      <c r="AO22" s="10">
         <v>3.22</v>
       </c>
-      <c r="AP22" s="15">
+      <c r="AP22" s="10">
         <v>8.19</v>
       </c>
-      <c r="AQ22" s="15">
+      <c r="AQ22" s="10">
         <v>4.4800000000000004</v>
       </c>
-      <c r="AR22" s="15">
+      <c r="AR22" s="10">
         <v>3.73</v>
       </c>
-      <c r="AS22" s="15">
+      <c r="AS22" s="10">
         <v>9.35</v>
       </c>
     </row>
-    <row r="23" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
-      <c r="B23" s="20" t="s">
+    <row r="23" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14"/>
+      <c r="B23" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="10">
         <v>2.04</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="10">
         <v>1.73</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="10">
         <v>3.6</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="10">
         <v>1.76</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="10">
         <v>1.51</v>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="10">
         <v>3.01</v>
       </c>
-      <c r="J23" s="15">
+      <c r="J23" s="10">
         <v>1.75</v>
       </c>
-      <c r="K23" s="15">
+      <c r="K23" s="10">
         <v>1.56</v>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="10">
         <v>2.78</v>
       </c>
-      <c r="M23" s="15">
+      <c r="M23" s="10">
         <v>2.2799999999999998</v>
       </c>
-      <c r="N23" s="15">
+      <c r="N23" s="10">
         <v>2.0699999999999998</v>
       </c>
-      <c r="O23" s="15">
+      <c r="O23" s="10">
         <v>3.42</v>
       </c>
-      <c r="P23" s="15">
+      <c r="P23" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q23" s="10">
         <v>1.9</v>
       </c>
-      <c r="R23" s="15">
+      <c r="R23" s="10">
         <v>3.75</v>
       </c>
-      <c r="S23" s="15">
+      <c r="S23" s="10">
         <v>2.16</v>
       </c>
-      <c r="T23" s="15">
+      <c r="T23" s="10">
         <v>1.81</v>
       </c>
-      <c r="U23" s="15">
+      <c r="U23" s="10">
         <v>4.03</v>
       </c>
-      <c r="V23" s="15">
+      <c r="V23" s="10">
         <v>2.37</v>
       </c>
-      <c r="W23" s="15">
+      <c r="W23" s="10">
         <v>2.1800000000000002</v>
       </c>
-      <c r="X23" s="15">
+      <c r="X23" s="10">
         <v>3.42</v>
       </c>
-      <c r="Y23" s="15">
+      <c r="Y23" s="10">
         <v>2.81</v>
       </c>
-      <c r="Z23" s="15">
+      <c r="Z23" s="10">
         <v>2.4300000000000002</v>
       </c>
-      <c r="AA23" s="15">
+      <c r="AA23" s="10">
         <v>4.93</v>
       </c>
-      <c r="AB23" s="15">
+      <c r="AB23" s="10">
         <v>2.98</v>
       </c>
-      <c r="AC23" s="15">
+      <c r="AC23" s="10">
         <v>2.63</v>
       </c>
-      <c r="AD23" s="15">
+      <c r="AD23" s="10">
         <v>5.09</v>
       </c>
-      <c r="AE23" s="15">
+      <c r="AE23" s="10">
         <v>3.16</v>
       </c>
-      <c r="AF23" s="15">
+      <c r="AF23" s="10">
         <v>2.5499999999999998</v>
       </c>
-      <c r="AG23" s="15">
+      <c r="AG23" s="10">
         <v>7.1</v>
       </c>
-      <c r="AH23" s="15">
+      <c r="AH23" s="10">
         <v>3.84</v>
       </c>
-      <c r="AI23" s="15">
+      <c r="AI23" s="10">
         <v>3.31</v>
       </c>
-      <c r="AJ23" s="15">
+      <c r="AJ23" s="10">
         <v>7.33</v>
       </c>
-      <c r="AK23" s="15">
+      <c r="AK23" s="10">
         <v>3.8</v>
       </c>
-      <c r="AL23" s="15">
+      <c r="AL23" s="10">
         <v>3.03</v>
       </c>
-      <c r="AM23" s="15">
+      <c r="AM23" s="10">
         <v>8.39</v>
       </c>
-      <c r="AN23" s="15">
+      <c r="AN23" s="10">
         <v>3.92</v>
       </c>
-      <c r="AO23" s="15">
+      <c r="AO23" s="10">
         <v>3.28</v>
       </c>
-      <c r="AP23" s="15">
+      <c r="AP23" s="10">
         <v>8.0299999999999994</v>
       </c>
-      <c r="AQ23" s="15">
+      <c r="AQ23" s="10">
         <v>4.01</v>
       </c>
-      <c r="AR23" s="15">
+      <c r="AR23" s="10">
         <v>3.27</v>
       </c>
-      <c r="AS23" s="15">
+      <c r="AS23" s="10">
         <v>9.18</v>
       </c>
     </row>
-    <row r="24" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="20" t="s">
+    <row r="24" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="10">
         <v>3.29</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="10">
         <v>2.31</v>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="10">
         <v>5.63</v>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="10">
         <v>2.74</v>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="10">
         <v>2.06</v>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="10">
         <v>4.43</v>
       </c>
-      <c r="J24" s="15">
+      <c r="J24" s="10">
         <v>2.6</v>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="10">
         <v>2.04</v>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="10">
         <v>4.1100000000000003</v>
       </c>
-      <c r="M24" s="15">
+      <c r="M24" s="10">
         <v>2.71</v>
       </c>
-      <c r="N24" s="15">
+      <c r="N24" s="10">
         <v>2.17</v>
       </c>
-      <c r="O24" s="15">
+      <c r="O24" s="10">
         <v>4.2300000000000004</v>
       </c>
-      <c r="P24" s="15">
+      <c r="P24" s="10">
         <v>3.15</v>
       </c>
-      <c r="Q24" s="15">
+      <c r="Q24" s="10">
         <v>2.5</v>
       </c>
-      <c r="R24" s="15">
+      <c r="R24" s="10">
         <v>5.0599999999999996</v>
       </c>
-      <c r="S24" s="15">
+      <c r="S24" s="10">
         <v>3.03</v>
       </c>
-      <c r="T24" s="15">
+      <c r="T24" s="10">
         <v>2.37</v>
       </c>
-      <c r="U24" s="15">
+      <c r="U24" s="10">
         <v>5.09</v>
       </c>
-      <c r="V24" s="15">
+      <c r="V24" s="10">
         <v>3.06</v>
       </c>
-      <c r="W24" s="15">
+      <c r="W24" s="10">
         <v>2.48</v>
       </c>
-      <c r="X24" s="15">
+      <c r="X24" s="10">
         <v>4.92</v>
       </c>
-      <c r="Y24" s="15">
+      <c r="Y24" s="10">
         <v>3.48</v>
       </c>
-      <c r="Z24" s="15">
+      <c r="Z24" s="10">
         <v>2.72</v>
       </c>
-      <c r="AA24" s="15">
+      <c r="AA24" s="10">
         <v>5.85</v>
       </c>
-      <c r="AB24" s="15">
+      <c r="AB24" s="10">
         <v>3.81</v>
       </c>
-      <c r="AC24" s="15">
+      <c r="AC24" s="10">
         <v>3.1</v>
       </c>
-      <c r="AD24" s="15">
+      <c r="AD24" s="10">
         <v>6.47</v>
       </c>
-      <c r="AE24" s="15">
+      <c r="AE24" s="10">
         <v>3.8</v>
       </c>
-      <c r="AF24" s="15">
+      <c r="AF24" s="10">
         <v>3.36</v>
       </c>
-      <c r="AG24" s="15">
+      <c r="AG24" s="10">
         <v>5.75</v>
       </c>
-      <c r="AH24" s="15">
+      <c r="AH24" s="10">
         <v>4.26</v>
       </c>
-      <c r="AI24" s="15">
+      <c r="AI24" s="10">
         <v>3.82</v>
       </c>
-      <c r="AJ24" s="15">
+      <c r="AJ24" s="10">
         <v>6.23</v>
       </c>
-      <c r="AK24" s="15">
+      <c r="AK24" s="10">
         <v>4.37</v>
       </c>
-      <c r="AL24" s="15">
+      <c r="AL24" s="10">
         <v>3.8</v>
       </c>
-      <c r="AM24" s="15">
+      <c r="AM24" s="10">
         <v>6.78</v>
       </c>
-      <c r="AN24" s="15">
+      <c r="AN24" s="10">
         <v>4.26</v>
       </c>
-      <c r="AO24" s="15">
+      <c r="AO24" s="10">
         <v>3.6</v>
       </c>
-      <c r="AP24" s="15">
+      <c r="AP24" s="10">
         <v>7.43</v>
       </c>
-      <c r="AQ24" s="15">
+      <c r="AQ24" s="10">
         <v>4.53</v>
       </c>
-      <c r="AR24" s="15">
+      <c r="AR24" s="10">
         <v>3.87</v>
       </c>
-      <c r="AS24" s="15">
+      <c r="AS24" s="10">
         <v>7.8</v>
       </c>
     </row>
-    <row r="25" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20" t="s">
+    <row r="25" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14"/>
+      <c r="B25" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="10">
         <v>3.57</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="10">
         <v>2.98</v>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="10">
         <v>4.62</v>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="10">
         <v>3.68</v>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="10">
         <v>3.28</v>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="10">
         <v>4.45</v>
       </c>
-      <c r="J25" s="15">
+      <c r="J25" s="10">
         <v>3.07</v>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="10">
         <v>2.64</v>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="10">
         <v>3.96</v>
       </c>
-      <c r="M25" s="15">
+      <c r="M25" s="10">
         <v>2.48</v>
       </c>
-      <c r="N25" s="15">
+      <c r="N25" s="10">
         <v>2.4900000000000002</v>
       </c>
-      <c r="O25" s="15">
+      <c r="O25" s="10">
         <v>2.46</v>
       </c>
-      <c r="P25" s="15">
+      <c r="P25" s="10">
         <v>2.77</v>
       </c>
-      <c r="Q25" s="15">
+      <c r="Q25" s="10">
         <v>2.77</v>
       </c>
-      <c r="R25" s="15">
+      <c r="R25" s="10">
         <v>2.77</v>
       </c>
-      <c r="S25" s="15">
+      <c r="S25" s="10">
         <v>2.85</v>
       </c>
-      <c r="T25" s="15">
+      <c r="T25" s="10">
         <v>2.33</v>
       </c>
-      <c r="U25" s="15">
+      <c r="U25" s="10">
         <v>4.25</v>
       </c>
-      <c r="V25" s="15">
+      <c r="V25" s="10">
         <v>2.8</v>
       </c>
-      <c r="W25" s="15">
+      <c r="W25" s="10">
         <v>2.81</v>
       </c>
-      <c r="X25" s="15">
+      <c r="X25" s="10">
         <v>2.77</v>
       </c>
-      <c r="Y25" s="15">
+      <c r="Y25" s="10">
         <v>2.5499999999999998</v>
       </c>
-      <c r="Z25" s="15">
+      <c r="Z25" s="10">
         <v>2.0099999999999998</v>
       </c>
-      <c r="AA25" s="15">
+      <c r="AA25" s="10">
         <v>4.05</v>
       </c>
-      <c r="AB25" s="15">
+      <c r="AB25" s="10">
         <v>2.56</v>
       </c>
-      <c r="AC25" s="15">
+      <c r="AC25" s="10">
         <v>2.42</v>
       </c>
-      <c r="AD25" s="15">
+      <c r="AD25" s="10">
         <v>3.01</v>
       </c>
-      <c r="AE25" s="15">
+      <c r="AE25" s="10">
         <v>2.65</v>
       </c>
-      <c r="AF25" s="15">
+      <c r="AF25" s="10">
         <v>2.4500000000000002</v>
       </c>
-      <c r="AG25" s="15">
+      <c r="AG25" s="10">
         <v>3.37</v>
       </c>
-      <c r="AH25" s="15">
+      <c r="AH25" s="10">
         <v>2.7</v>
       </c>
-      <c r="AI25" s="15">
+      <c r="AI25" s="10">
         <v>2.25</v>
       </c>
-      <c r="AJ25" s="15">
+      <c r="AJ25" s="10">
         <v>4.3600000000000003</v>
       </c>
-      <c r="AK25" s="15">
+      <c r="AK25" s="10">
         <v>3.52</v>
       </c>
-      <c r="AL25" s="15">
+      <c r="AL25" s="10">
         <v>3.57</v>
       </c>
-      <c r="AM25" s="15">
+      <c r="AM25" s="10">
         <v>3.38</v>
       </c>
-      <c r="AN25" s="15">
+      <c r="AN25" s="10">
         <v>3.53</v>
       </c>
-      <c r="AO25" s="15">
+      <c r="AO25" s="10">
         <v>3.22</v>
       </c>
-      <c r="AP25" s="15">
+      <c r="AP25" s="10">
         <v>4.71</v>
       </c>
-      <c r="AQ25" s="15">
+      <c r="AQ25" s="10">
         <v>4.24</v>
       </c>
-      <c r="AR25" s="15">
+      <c r="AR25" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="AS25" s="15">
+      <c r="AS25" s="10">
         <v>3.63</v>
       </c>
     </row>
-    <row r="26" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
-      <c r="B26" s="20" t="s">
+    <row r="26" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14"/>
+      <c r="B26" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="10">
         <v>3.36</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="10">
         <v>2.2400000000000002</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="10">
         <v>5.78</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="10">
         <v>2.91</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="10">
         <v>2.19</v>
       </c>
-      <c r="I26" s="15">
+      <c r="I26" s="10">
         <v>4.5199999999999996</v>
       </c>
-      <c r="J26" s="15">
+      <c r="J26" s="10">
         <v>2.1</v>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="10">
         <v>1.78</v>
       </c>
-      <c r="L26" s="15">
+      <c r="L26" s="10">
         <v>2.85</v>
       </c>
-      <c r="M26" s="15">
+      <c r="M26" s="10">
         <v>2.68</v>
       </c>
-      <c r="N26" s="15">
+      <c r="N26" s="10">
         <v>2.3199999999999998</v>
       </c>
-      <c r="O26" s="15">
+      <c r="O26" s="10">
         <v>3.55</v>
       </c>
-      <c r="P26" s="15">
+      <c r="P26" s="10">
         <v>2.46</v>
       </c>
-      <c r="Q26" s="15">
+      <c r="Q26" s="10">
         <v>1.92</v>
       </c>
-      <c r="R26" s="15">
+      <c r="R26" s="10">
         <v>3.88</v>
       </c>
-      <c r="S26" s="15">
+      <c r="S26" s="10">
         <v>2.41</v>
       </c>
-      <c r="T26" s="15">
+      <c r="T26" s="10">
         <v>2.14</v>
       </c>
-      <c r="U26" s="15">
+      <c r="U26" s="10">
         <v>3.09</v>
       </c>
-      <c r="V26" s="15">
+      <c r="V26" s="10">
         <v>2.98</v>
       </c>
-      <c r="W26" s="15">
+      <c r="W26" s="10">
         <v>2.5099999999999998</v>
       </c>
-      <c r="X26" s="15">
+      <c r="X26" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="Y26" s="15">
+      <c r="Y26" s="10">
         <v>3.07</v>
       </c>
-      <c r="Z26" s="15">
+      <c r="Z26" s="10">
         <v>2.75</v>
       </c>
-      <c r="AA26" s="15">
+      <c r="AA26" s="10">
         <v>3.84</v>
       </c>
-      <c r="AB26" s="15">
+      <c r="AB26" s="10">
         <v>3.56</v>
       </c>
-      <c r="AC26" s="15">
+      <c r="AC26" s="10">
         <v>3.45</v>
       </c>
-      <c r="AD26" s="15">
+      <c r="AD26" s="10">
         <v>3.9</v>
       </c>
-      <c r="AE26" s="15">
+      <c r="AE26" s="10">
         <v>3.37</v>
       </c>
-      <c r="AF26" s="15">
+      <c r="AF26" s="10">
         <v>2.6</v>
       </c>
-      <c r="AG26" s="15">
+      <c r="AG26" s="10">
         <v>5.88</v>
       </c>
-      <c r="AH26" s="15">
+      <c r="AH26" s="10">
         <v>3.99</v>
       </c>
-      <c r="AI26" s="15">
+      <c r="AI26" s="10">
         <v>3.65</v>
       </c>
-      <c r="AJ26" s="15">
+      <c r="AJ26" s="10">
         <v>5.13</v>
       </c>
-      <c r="AK26" s="15">
+      <c r="AK26" s="10">
         <v>3.76</v>
       </c>
-      <c r="AL26" s="15">
+      <c r="AL26" s="10">
         <v>3.57</v>
       </c>
-      <c r="AM26" s="15">
+      <c r="AM26" s="10">
         <v>4.3099999999999996</v>
       </c>
-      <c r="AN26" s="15">
+      <c r="AN26" s="10">
         <v>3.82</v>
       </c>
-      <c r="AO26" s="15">
+      <c r="AO26" s="10">
         <v>3.42</v>
       </c>
-      <c r="AP26" s="15">
+      <c r="AP26" s="10">
         <v>5.15</v>
       </c>
-      <c r="AQ26" s="15">
+      <c r="AQ26" s="10">
         <v>4.84</v>
       </c>
-      <c r="AR26" s="15">
+      <c r="AR26" s="10">
         <v>4.74</v>
       </c>
-      <c r="AS26" s="15">
+      <c r="AS26" s="10">
         <v>5.2</v>
       </c>
     </row>
-    <row r="27" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
-      <c r="B27" s="20" t="s">
+    <row r="27" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="14"/>
+      <c r="B27" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="10">
         <v>2.5</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="10">
         <v>1.83</v>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="10">
         <v>3.79</v>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="10">
         <v>2.5</v>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="10">
         <v>1.39</v>
       </c>
-      <c r="I27" s="15">
+      <c r="I27" s="10">
         <v>4.53</v>
       </c>
-      <c r="J27" s="15">
+      <c r="J27" s="10">
         <v>1.91</v>
       </c>
-      <c r="K27" s="15">
+      <c r="K27" s="10">
         <v>1.32</v>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="10">
         <v>3.11</v>
       </c>
-      <c r="M27" s="15">
+      <c r="M27" s="10">
         <v>1.64</v>
       </c>
-      <c r="N27" s="15">
+      <c r="N27" s="10">
         <v>1.28</v>
       </c>
-      <c r="O27" s="15">
+      <c r="O27" s="10">
         <v>2.39</v>
       </c>
-      <c r="P27" s="15">
+      <c r="P27" s="10">
         <v>2.48</v>
       </c>
-      <c r="Q27" s="15">
+      <c r="Q27" s="10">
         <v>2.2400000000000002</v>
       </c>
-      <c r="R27" s="15">
+      <c r="R27" s="10">
         <v>3.03</v>
       </c>
-      <c r="S27" s="15">
+      <c r="S27" s="10">
         <v>2.04</v>
       </c>
-      <c r="T27" s="15">
+      <c r="T27" s="10">
         <v>1.52</v>
       </c>
-      <c r="U27" s="15">
+      <c r="U27" s="10">
         <v>3.29</v>
       </c>
-      <c r="V27" s="15">
+      <c r="V27" s="10">
         <v>1.92</v>
       </c>
-      <c r="W27" s="15">
+      <c r="W27" s="10">
         <v>1.3</v>
       </c>
-      <c r="X27" s="15">
+      <c r="X27" s="10">
         <v>3.4</v>
       </c>
-      <c r="Y27" s="15">
+      <c r="Y27" s="10">
         <v>2.77</v>
       </c>
-      <c r="Z27" s="15">
+      <c r="Z27" s="10">
         <v>2.11</v>
       </c>
-      <c r="AA27" s="15">
+      <c r="AA27" s="10">
         <v>4.41</v>
       </c>
-      <c r="AB27" s="15">
+      <c r="AB27" s="10">
         <v>2.5299999999999998</v>
       </c>
-      <c r="AC27" s="15">
+      <c r="AC27" s="10">
         <v>2</v>
       </c>
-      <c r="AD27" s="15">
+      <c r="AD27" s="10">
         <v>4.16</v>
       </c>
-      <c r="AE27" s="15">
+      <c r="AE27" s="10">
         <v>3.15</v>
       </c>
-      <c r="AF27" s="15">
+      <c r="AF27" s="10">
         <v>2.71</v>
       </c>
-      <c r="AG27" s="15">
+      <c r="AG27" s="10">
         <v>4.66</v>
       </c>
-      <c r="AH27" s="15">
+      <c r="AH27" s="10">
         <v>3.11</v>
       </c>
-      <c r="AI27" s="15">
+      <c r="AI27" s="10">
         <v>2.77</v>
       </c>
-      <c r="AJ27" s="15">
+      <c r="AJ27" s="10">
         <v>4.38</v>
       </c>
-      <c r="AK27" s="15">
+      <c r="AK27" s="10">
         <v>3.34</v>
       </c>
-      <c r="AL27" s="15">
+      <c r="AL27" s="10">
         <v>3.08</v>
       </c>
-      <c r="AM27" s="15">
+      <c r="AM27" s="10">
         <v>4.37</v>
       </c>
-      <c r="AN27" s="15">
+      <c r="AN27" s="10">
         <v>3.13</v>
       </c>
-      <c r="AO27" s="15">
+      <c r="AO27" s="10">
         <v>2.99</v>
       </c>
-      <c r="AP27" s="15">
+      <c r="AP27" s="10">
         <v>3.79</v>
       </c>
-      <c r="AQ27" s="15">
+      <c r="AQ27" s="10">
         <v>3.74</v>
       </c>
-      <c r="AR27" s="15">
+      <c r="AR27" s="10">
         <v>3.28</v>
       </c>
-      <c r="AS27" s="15">
+      <c r="AS27" s="10">
         <v>5.9</v>
       </c>
     </row>
-    <row r="28" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="19"/>
-      <c r="B28" s="20" t="s">
+    <row r="28" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="14"/>
+      <c r="B28" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="10">
         <v>1.78</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="10">
         <v>0.95</v>
       </c>
-      <c r="F28" s="15">
+      <c r="F28" s="10">
         <v>3.73</v>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="10">
         <v>1.78</v>
       </c>
-      <c r="H28" s="15">
+      <c r="H28" s="10">
         <v>1.03</v>
       </c>
-      <c r="I28" s="15">
+      <c r="I28" s="10">
         <v>3.74</v>
       </c>
-      <c r="J28" s="15">
+      <c r="J28" s="10">
         <v>1.67</v>
       </c>
-      <c r="K28" s="15">
+      <c r="K28" s="10">
         <v>1.44</v>
       </c>
-      <c r="L28" s="15">
+      <c r="L28" s="10">
         <v>2.38</v>
       </c>
-      <c r="M28" s="15">
+      <c r="M28" s="10">
         <v>1.48</v>
       </c>
-      <c r="N28" s="15">
+      <c r="N28" s="10">
         <v>1.06</v>
       </c>
-      <c r="O28" s="15">
+      <c r="O28" s="10">
         <v>2.84</v>
       </c>
-      <c r="P28" s="15">
+      <c r="P28" s="10">
         <v>1.86</v>
       </c>
-      <c r="Q28" s="15">
+      <c r="Q28" s="10">
         <v>1.49</v>
       </c>
-      <c r="R28" s="15">
+      <c r="R28" s="10">
         <v>3.24</v>
       </c>
-      <c r="S28" s="15">
+      <c r="S28" s="10">
         <v>1.36</v>
       </c>
-      <c r="T28" s="15">
+      <c r="T28" s="10">
         <v>1.02</v>
       </c>
-      <c r="U28" s="15">
+      <c r="U28" s="10">
         <v>2.86</v>
       </c>
-      <c r="V28" s="15">
+      <c r="V28" s="10">
         <v>1.84</v>
       </c>
-      <c r="W28" s="15">
+      <c r="W28" s="10">
         <v>1.51</v>
       </c>
-      <c r="X28" s="15">
+      <c r="X28" s="10">
         <v>3.33</v>
       </c>
-      <c r="Y28" s="15">
+      <c r="Y28" s="10">
         <v>2.09</v>
       </c>
-      <c r="Z28" s="15">
+      <c r="Z28" s="10">
         <v>1.7</v>
       </c>
-      <c r="AA28" s="15">
+      <c r="AA28" s="10">
         <v>4.01</v>
       </c>
-      <c r="AB28" s="15">
+      <c r="AB28" s="10">
         <v>2.02</v>
       </c>
-      <c r="AC28" s="15">
+      <c r="AC28" s="10">
         <v>1.91</v>
       </c>
-      <c r="AD28" s="15">
+      <c r="AD28" s="10">
         <v>2.69</v>
       </c>
-      <c r="AE28" s="15">
+      <c r="AE28" s="10">
         <v>3.03</v>
       </c>
-      <c r="AF28" s="15">
+      <c r="AF28" s="10">
         <v>2.79</v>
       </c>
-      <c r="AG28" s="15">
+      <c r="AG28" s="10">
         <v>4.54</v>
       </c>
-      <c r="AH28" s="15">
+      <c r="AH28" s="10">
         <v>3.01</v>
       </c>
-      <c r="AI28" s="15">
+      <c r="AI28" s="10">
         <v>2.74</v>
       </c>
-      <c r="AJ28" s="15">
+      <c r="AJ28" s="10">
         <v>4.67</v>
       </c>
-      <c r="AK28" s="15">
+      <c r="AK28" s="10">
         <v>3.18</v>
       </c>
-      <c r="AL28" s="15">
+      <c r="AL28" s="10">
         <v>2.94</v>
       </c>
-      <c r="AM28" s="15">
+      <c r="AM28" s="10">
         <v>4.55</v>
       </c>
-      <c r="AN28" s="15">
+      <c r="AN28" s="10">
         <v>3.38</v>
       </c>
-      <c r="AO28" s="15">
+      <c r="AO28" s="10">
         <v>3.03</v>
       </c>
-      <c r="AP28" s="15">
+      <c r="AP28" s="10">
         <v>5.5</v>
       </c>
-      <c r="AQ28" s="15">
+      <c r="AQ28" s="10">
         <v>3.92</v>
       </c>
-      <c r="AR28" s="15">
+      <c r="AR28" s="10">
         <v>3.65</v>
       </c>
-      <c r="AS28" s="15">
+      <c r="AS28" s="10">
         <v>5.58</v>
       </c>
     </row>
-    <row r="29" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="19"/>
-      <c r="B29" s="20" t="s">
+    <row r="29" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="14"/>
+      <c r="B29" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="10">
         <v>1.34</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="10">
         <v>1.26</v>
       </c>
-      <c r="F29" s="15">
+      <c r="F29" s="10">
         <v>1.73</v>
       </c>
-      <c r="G29" s="15">
+      <c r="G29" s="10">
         <v>1.38</v>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="10">
         <v>1.1100000000000001</v>
       </c>
-      <c r="I29" s="15">
+      <c r="I29" s="10">
         <v>2.62</v>
       </c>
-      <c r="J29" s="15">
+      <c r="J29" s="10">
         <v>1.24</v>
       </c>
-      <c r="K29" s="15">
+      <c r="K29" s="10">
         <v>1.1200000000000001</v>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="10">
         <v>1.93</v>
       </c>
-      <c r="M29" s="15">
+      <c r="M29" s="10">
         <v>1.46</v>
       </c>
-      <c r="N29" s="15">
+      <c r="N29" s="10">
         <v>1.35</v>
       </c>
-      <c r="O29" s="15">
+      <c r="O29" s="10">
         <v>2.08</v>
       </c>
-      <c r="P29" s="15">
+      <c r="P29" s="10">
         <v>1.5</v>
       </c>
-      <c r="Q29" s="15">
+      <c r="Q29" s="10">
         <v>1.33</v>
       </c>
-      <c r="R29" s="15">
+      <c r="R29" s="10">
         <v>2.4300000000000002</v>
       </c>
-      <c r="S29" s="15">
+      <c r="S29" s="10">
         <v>1.35</v>
       </c>
-      <c r="T29" s="15">
+      <c r="T29" s="10">
         <v>1.27</v>
       </c>
-      <c r="U29" s="15">
+      <c r="U29" s="10">
         <v>1.84</v>
       </c>
-      <c r="V29" s="15">
+      <c r="V29" s="10">
         <v>1.58</v>
       </c>
-      <c r="W29" s="15">
+      <c r="W29" s="10">
         <v>1.55</v>
       </c>
-      <c r="X29" s="15">
+      <c r="X29" s="10">
         <v>1.78</v>
       </c>
-      <c r="Y29" s="15">
+      <c r="Y29" s="10">
         <v>1.94</v>
       </c>
-      <c r="Z29" s="15">
+      <c r="Z29" s="10">
         <v>1.75</v>
       </c>
-      <c r="AA29" s="15">
+      <c r="AA29" s="10">
         <v>2.97</v>
       </c>
-      <c r="AB29" s="15">
+      <c r="AB29" s="10">
         <v>1.95</v>
       </c>
-      <c r="AC29" s="15">
+      <c r="AC29" s="10">
         <v>1.67</v>
       </c>
-      <c r="AD29" s="15">
+      <c r="AD29" s="10">
         <v>3.54</v>
       </c>
-      <c r="AE29" s="15">
+      <c r="AE29" s="10">
         <v>2.09</v>
       </c>
-      <c r="AF29" s="15">
+      <c r="AF29" s="10">
         <v>1.95</v>
       </c>
-      <c r="AG29" s="15">
+      <c r="AG29" s="10">
         <v>2.89</v>
       </c>
-      <c r="AH29" s="15">
+      <c r="AH29" s="10">
         <v>2.33</v>
       </c>
-      <c r="AI29" s="15">
+      <c r="AI29" s="10">
         <v>2.14</v>
       </c>
-      <c r="AJ29" s="15">
+      <c r="AJ29" s="10">
         <v>3.47</v>
       </c>
-      <c r="AK29" s="15">
+      <c r="AK29" s="10">
         <v>2.6</v>
       </c>
-      <c r="AL29" s="15">
+      <c r="AL29" s="10">
         <v>2.56</v>
       </c>
-      <c r="AM29" s="15">
+      <c r="AM29" s="10">
         <v>2.86</v>
       </c>
-      <c r="AN29" s="15">
+      <c r="AN29" s="10">
         <v>2.5099999999999998</v>
       </c>
-      <c r="AO29" s="15">
+      <c r="AO29" s="10">
         <v>2.16</v>
       </c>
-      <c r="AP29" s="15">
+      <c r="AP29" s="10">
         <v>4.74</v>
       </c>
-      <c r="AQ29" s="15">
+      <c r="AQ29" s="10">
         <v>3.1</v>
       </c>
-      <c r="AR29" s="15">
+      <c r="AR29" s="10">
         <v>2.56</v>
       </c>
-      <c r="AS29" s="15">
+      <c r="AS29" s="10">
         <v>6.58</v>
       </c>
     </row>
-    <row r="30" spans="1:45" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="19"/>
-      <c r="B30" s="20" t="s">
+    <row r="30" spans="1:45" s="17" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="14"/>
+      <c r="B30" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="10">
         <v>2.39</v>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="10">
         <v>1.73</v>
       </c>
-      <c r="F30" s="15">
+      <c r="F30" s="10">
         <v>4.03</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="10">
         <v>2.35</v>
       </c>
-      <c r="H30" s="15">
+      <c r="H30" s="10">
         <v>1.67</v>
       </c>
-      <c r="I30" s="15">
+      <c r="I30" s="10">
         <v>4.08</v>
       </c>
-      <c r="J30" s="15">
+      <c r="J30" s="10">
         <v>1.92</v>
       </c>
-      <c r="K30" s="15">
+      <c r="K30" s="10">
         <v>1.57</v>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="10">
         <v>2.92</v>
       </c>
-      <c r="M30" s="15">
+      <c r="M30" s="10">
         <v>1.9</v>
       </c>
-      <c r="N30" s="15">
+      <c r="N30" s="10">
         <v>1.63</v>
       </c>
-      <c r="O30" s="15">
+      <c r="O30" s="10">
         <v>2.71</v>
       </c>
-      <c r="P30" s="15">
+      <c r="P30" s="10">
         <v>2.17</v>
       </c>
-      <c r="Q30" s="15">
+      <c r="Q30" s="10">
         <v>1.86</v>
       </c>
-      <c r="R30" s="15">
+      <c r="R30" s="10">
         <v>3.14</v>
       </c>
-      <c r="S30" s="15">
+      <c r="S30" s="10">
         <v>1.91</v>
       </c>
-      <c r="T30" s="15">
+      <c r="T30" s="10">
         <v>1.55</v>
       </c>
-      <c r="U30" s="15">
+      <c r="U30" s="10">
         <v>3.13</v>
       </c>
-      <c r="V30" s="15">
+      <c r="V30" s="10">
         <v>2.15</v>
       </c>
-      <c r="W30" s="15">
+      <c r="W30" s="10">
         <v>1.85</v>
       </c>
-      <c r="X30" s="15">
+      <c r="X30" s="10">
         <v>3.19</v>
       </c>
-      <c r="Y30" s="15">
+      <c r="Y30" s="10">
         <v>2.4300000000000002</v>
       </c>
-      <c r="Z30" s="15">
+      <c r="Z30" s="10">
         <v>2</v>
       </c>
-      <c r="AA30" s="15">
+      <c r="AA30" s="10">
         <v>3.91</v>
       </c>
-      <c r="AB30" s="15">
+      <c r="AB30" s="10">
         <v>2.46</v>
       </c>
-      <c r="AC30" s="15">
+      <c r="AC30" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="AD30" s="15">
+      <c r="AD30" s="10">
         <v>3.5</v>
       </c>
-      <c r="AE30" s="15">
+      <c r="AE30" s="10">
         <v>2.85</v>
       </c>
-      <c r="AF30" s="15">
+      <c r="AF30" s="10">
         <v>2.5</v>
       </c>
-      <c r="AG30" s="15">
+      <c r="AG30" s="10">
         <v>4.37</v>
       </c>
-      <c r="AH30" s="15">
+      <c r="AH30" s="10">
         <v>3.01</v>
       </c>
-      <c r="AI30" s="15">
+      <c r="AI30" s="10">
         <v>2.69</v>
       </c>
-      <c r="AJ30" s="15">
+      <c r="AJ30" s="10">
         <v>4.45</v>
       </c>
-      <c r="AK30" s="15">
+      <c r="AK30" s="10">
         <v>3.25</v>
       </c>
-      <c r="AL30" s="15">
+      <c r="AL30" s="10">
         <v>3.08</v>
       </c>
-      <c r="AM30" s="15">
+      <c r="AM30" s="10">
         <v>3.97</v>
       </c>
-      <c r="AN30" s="15">
+      <c r="AN30" s="10">
         <v>3.26</v>
       </c>
-      <c r="AO30" s="15">
+      <c r="AO30" s="10">
         <v>2.94</v>
       </c>
-      <c r="AP30" s="15">
+      <c r="AP30" s="10">
         <v>4.79</v>
       </c>
-      <c r="AQ30" s="15">
+      <c r="AQ30" s="10">
         <v>3.93</v>
       </c>
-      <c r="AR30" s="15">
+      <c r="AR30" s="10">
         <v>3.65</v>
       </c>
-      <c r="AS30" s="15">
+      <c r="AS30" s="10">
         <v>5.32</v>
       </c>
     </row>
     <row r="31" spans="1:45" x14ac:dyDescent="0.25">
       <c r="B31" s="7"/>
     </row>
-    <row r="32" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="B32" s="29" t="s">
+    <row r="32" spans="1:45" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+    </row>
+    <row r="33" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B34" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="18"/>
+    </row>
+    <row r="35" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="29"/>
-      <c r="L32" s="29"/>
-      <c r="M32" s="29"/>
-      <c r="N32" s="29"/>
-      <c r="O32" s="29"/>
-      <c r="P32" s="29"/>
-      <c r="Q32" s="29"/>
-      <c r="R32" s="29"/>
-      <c r="S32" s="29"/>
-      <c r="T32" s="29"/>
-      <c r="U32" s="29"/>
-      <c r="V32" s="29"/>
-      <c r="W32" s="29"/>
-      <c r="X32" s="29"/>
-      <c r="Y32" s="29"/>
-      <c r="Z32" s="29"/>
-      <c r="AA32" s="29"/>
-      <c r="AB32" s="29"/>
-      <c r="AC32" s="29"/>
-      <c r="AD32" s="29"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
     </row>
-    <row r="33" spans="2:30" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="30" t="s">
+    <row r="36" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="9"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+    </row>
+    <row r="37" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="30"/>
-      <c r="P33" s="30"/>
-      <c r="Q33" s="30"/>
-      <c r="R33" s="30"/>
-      <c r="S33" s="30"/>
-      <c r="T33" s="30"/>
-      <c r="U33" s="30"/>
-      <c r="V33" s="30"/>
-      <c r="W33" s="30"/>
-      <c r="X33" s="30"/>
-      <c r="Y33" s="30"/>
-      <c r="Z33" s="30"/>
-      <c r="AA33" s="30"/>
-      <c r="AB33" s="30"/>
-      <c r="AC33" s="30"/>
-      <c r="AD33" s="30"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
     </row>
-    <row r="34" spans="2:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="31" t="s">
+    <row r="38" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+    </row>
+    <row r="39" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="31"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
     </row>
-    <row r="35" spans="2:30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="10" t="s">
+    <row r="40" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
+      <c r="M40" s="8"/>
+    </row>
+    <row r="41" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="11"/>
-      <c r="O35" s="11"/>
-      <c r="P35" s="11"/>
-      <c r="Q35" s="11"/>
-      <c r="R35" s="11"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="8"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="8"/>
+      <c r="M41" s="8"/>
     </row>
-    <row r="36" spans="2:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11"/>
-      <c r="O36" s="11"/>
-      <c r="P36" s="11"/>
-      <c r="Q36" s="11"/>
-      <c r="R36" s="11"/>
-      <c r="S36" s="11"/>
-      <c r="T36" s="11"/>
-      <c r="U36" s="11"/>
-      <c r="V36" s="11"/>
-      <c r="W36" s="11"/>
-      <c r="X36" s="11"/>
-      <c r="Y36" s="11"/>
-      <c r="Z36" s="11"/>
-      <c r="AA36" s="11"/>
-      <c r="AB36" s="11"/>
-      <c r="AC36" s="11"/>
-      <c r="AD36" s="11"/>
-    </row>
-    <row r="37" spans="2:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="11" t="s">
+    <row r="42" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="11"/>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
-      <c r="O37" s="11"/>
-      <c r="P37" s="11"/>
-      <c r="Q37" s="11"/>
-      <c r="R37" s="11"/>
-      <c r="S37" s="11"/>
-      <c r="T37" s="11"/>
-      <c r="U37" s="11"/>
-      <c r="V37" s="11"/>
-      <c r="W37" s="11"/>
-      <c r="X37" s="11"/>
-      <c r="Y37" s="11"/>
-      <c r="Z37" s="11"/>
-      <c r="AA37" s="11"/>
-      <c r="AB37" s="11"/>
-      <c r="AC37" s="11"/>
-      <c r="AD37" s="11"/>
-    </row>
-    <row r="39" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B39" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="40" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B40" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="41" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B41" s="13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="42" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B42" s="14" t="s">
-        <v>34</v>
-      </c>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="8"/>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="8"/>
+      <c r="M42" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="B32:AD32"/>
-    <mergeCell ref="B33:AD33"/>
-    <mergeCell ref="B34:R34"/>
-    <mergeCell ref="AN8:AN10"/>
-    <mergeCell ref="AO8:AO9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="W10:X10"/>
-    <mergeCell ref="AH8:AH10"/>
-    <mergeCell ref="AL8:AL9"/>
-    <mergeCell ref="AM8:AM9"/>
-    <mergeCell ref="AI10:AJ10"/>
-    <mergeCell ref="AL10:AM10"/>
-    <mergeCell ref="AO10:AP10"/>
-    <mergeCell ref="AP8:AP9"/>
-    <mergeCell ref="AE8:AE10"/>
-    <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="AI8:AI9"/>
-    <mergeCell ref="AJ8:AJ9"/>
-    <mergeCell ref="AK8:AK10"/>
+    <mergeCell ref="B32:M32"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="B34:M34"/>
+    <mergeCell ref="AS8:AS9"/>
+    <mergeCell ref="AR10:AS10"/>
+    <mergeCell ref="D11:AS11"/>
+    <mergeCell ref="AK7:AM7"/>
+    <mergeCell ref="AN7:AP7"/>
+    <mergeCell ref="M7:O7"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="V7:X7"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="B6:B11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J6:AS6"/>
+    <mergeCell ref="AQ7:AS7"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AR8:AR9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="Y7:AA7"/>
+    <mergeCell ref="AB7:AD7"/>
+    <mergeCell ref="AE7:AG7"/>
+    <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q9"/>
     <mergeCell ref="R8:R9"/>
     <mergeCell ref="S8:S10"/>
     <mergeCell ref="T8:T9"/>
@@ -4211,47 +4195,31 @@
     <mergeCell ref="AB8:AB10"/>
     <mergeCell ref="AC8:AC9"/>
     <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="B6:B11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J6:AS6"/>
-    <mergeCell ref="AQ7:AS7"/>
-    <mergeCell ref="AQ8:AQ10"/>
-    <mergeCell ref="AR8:AR9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="Y7:AA7"/>
-    <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="AE7:AG7"/>
-    <mergeCell ref="AH7:AJ7"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="AS8:AS9"/>
-    <mergeCell ref="AR10:AS10"/>
-    <mergeCell ref="D11:AS11"/>
-    <mergeCell ref="AK7:AM7"/>
-    <mergeCell ref="AN7:AP7"/>
-    <mergeCell ref="M7:O7"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="V7:X7"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="AL10:AM10"/>
+    <mergeCell ref="AO10:AP10"/>
+    <mergeCell ref="AP8:AP9"/>
+    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="AF8:AF9"/>
+    <mergeCell ref="AI8:AI9"/>
+    <mergeCell ref="AJ8:AJ9"/>
+    <mergeCell ref="AK8:AK10"/>
+    <mergeCell ref="AN8:AN10"/>
+    <mergeCell ref="AO8:AO9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="W10:X10"/>
+    <mergeCell ref="AH8:AH10"/>
+    <mergeCell ref="AL8:AL9"/>
+    <mergeCell ref="AM8:AM9"/>
+    <mergeCell ref="AI10:AJ10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B42" r:id="rId1" xr:uid="{F94324D3-9937-4F3E-A4F8-7AD7EC469BFB}"/>
-    <hyperlink ref="B35" r:id="rId2" xr:uid="{355D418E-7D08-4C2B-8B23-527CF3D655B2}"/>
+    <hyperlink ref="B35" r:id="rId1" xr:uid="{F43AA942-BDA1-449F-A14A-48D41A2BCD14}"/>
+    <hyperlink ref="B42" r:id="rId2" xr:uid="{E2864563-FDCA-4F3A-BD38-E53A3A703121}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>